<commit_message>
Refresh complete Gujjar Transport project
</commit_message>
<xml_diff>
--- a/verification/report-samples/combined-multipage.xlsx
+++ b/verification/report-samples/combined-multipage.xlsx
@@ -7,7 +7,7 @@
     <sheet sheetId="1" name="Report" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A1:$CF130</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A1:$CF126</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$12</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="175">
   <si>
     <t>Gujjar Brother Transport — TEST DATA ONLY</t>
   </si>
@@ -26,7 +26,7 @@
     <t>CYCLE INCOME DETAIL · TEST accounting period</t>
   </si>
   <si>
-    <t>2026-01-01 to 2026-12-31 · PKR · 2026-10-06T19:37:03.339+00:00</t>
+    <t>2026-01-01 to 2026-12-31 · PKR · 2026-10-11T16:34:22.859+00:00</t>
   </si>
   <si>
     <t>INCOMPLETE — missing mappings/sources; review notes.</t>
@@ -89,7 +89,7 @@
     <t>Diesel (Price)</t>
   </si>
   <si>
-    <t>Chln</t>
+    <t>Punjab Police</t>
   </si>
   <si>
     <t>Toll Plaza</t>
@@ -98,66 +98,66 @@
     <t>Food</t>
   </si>
   <si>
-    <t>inm</t>
-  </si>
-  <si>
-    <t>Other Exp.</t>
-  </si>
-  <si>
-    <t>Mobil Oil</t>
-  </si>
-  <si>
-    <t>Driver com</t>
-  </si>
-  <si>
-    <t>Total Exp.</t>
-  </si>
-  <si>
-    <t>Profit Loss</t>
-  </si>
-  <si>
-    <t>Travl (km)</t>
-  </si>
-  <si>
-    <t>Diesel (Ltr)</t>
-  </si>
-  <si>
-    <t>Avg Km/L</t>
+    <t>Inam / reward</t>
+  </si>
+  <si>
+    <t>Other expense</t>
+  </si>
+  <si>
+    <t>Engine oil</t>
+  </si>
+  <si>
+    <t>Driver cycle commission</t>
+  </si>
+  <si>
+    <t>Total expense</t>
+  </si>
+  <si>
+    <t>Profit / loss</t>
+  </si>
+  <si>
+    <t>Travel (km)</t>
+  </si>
+  <si>
+    <t>Diesel (L)</t>
+  </si>
+  <si>
+    <t>Average (km/L)</t>
+  </si>
+  <si>
+    <t>TEST gearbox structured invoice item</t>
+  </si>
+  <si>
+    <t>TEST multi-page route 0</t>
+  </si>
+  <si>
+    <t>TEST cabin structured invoice item</t>
+  </si>
+  <si>
+    <t>TEST multi-page route 1</t>
+  </si>
+  <si>
+    <t>TEST engine structured invoice item</t>
+  </si>
+  <si>
+    <t>TEST multi-page route 2</t>
   </si>
   <si>
     <t>TEST body structured invoice item</t>
   </si>
   <si>
-    <t>TEST multi-page route 0</t>
-  </si>
-  <si>
-    <t>TEST engine structured invoice item</t>
-  </si>
-  <si>
-    <t>TEST multi-page route 1</t>
+    <t>TEST multi-page route 3</t>
   </si>
   <si>
     <t>TEST oil_change structured invoice item</t>
   </si>
   <si>
-    <t>TEST multi-page route 2</t>
-  </si>
-  <si>
-    <t>TEST gearbox structured invoice item</t>
-  </si>
-  <si>
-    <t>TEST multi-page route 3</t>
+    <t>TEST multi-page route 4</t>
   </si>
   <si>
     <t>TEST tyres structured invoice item</t>
   </si>
   <si>
-    <t>TEST multi-page route 4</t>
-  </si>
-  <si>
-    <t>TEST cabin structured invoice item</t>
-  </si>
-  <si>
     <t>TEST multi-page route 5</t>
   </si>
   <si>
@@ -431,9 +431,6 @@
     <t>Monthly Maintenance</t>
   </si>
   <si>
-    <t>Driver Commission</t>
-  </si>
-  <si>
     <t>TRACKER</t>
   </si>
   <si>
@@ -449,7 +446,7 @@
     <t>Driver settlement</t>
   </si>
   <si>
-    <t>Dr.Name</t>
+    <t>Driver name</t>
   </si>
   <si>
     <t>Driver Sale</t>
@@ -467,7 +464,7 @@
     <t>Salary Advance</t>
   </si>
   <si>
-    <t>Loan Install.</t>
+    <t>Loan installment</t>
   </si>
   <si>
     <t>Irresponsible Vehicle loss</t>
@@ -485,64 +482,60 @@
     <t>Total Loan</t>
   </si>
   <si>
-    <t>Loan Return</t>
-  </si>
-  <si>
-    <t>Loan left</t>
+    <t>Loan repaid</t>
+  </si>
+  <si>
+    <t>Loan balance</t>
+  </si>
+  <si>
+    <t>ENGINE</t>
+  </si>
+  <si>
+    <t>GEAR</t>
+  </si>
+  <si>
+    <t>BODY / CABIN</t>
+  </si>
+  <si>
+    <t>TYRES</t>
+  </si>
+  <si>
+    <t>TEST unposted engine work detail</t>
+  </si>
+  <si>
+    <t>TEST unposted gearbox work detail</t>
+  </si>
+  <si>
+    <t>TEST unposted tyres work detail</t>
+  </si>
+  <si>
+    <t>Total Bill</t>
+  </si>
+  <si>
+    <t>TEST unposted body work detail</t>
+  </si>
+  <si>
+    <t>TEST unposted cabin work detail</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>DRIVER SIGN</t>
-  </si>
-  <si>
-    <t>DRIVER THUMB</t>
-  </si>
-  <si>
-    <t>PAID BY</t>
-  </si>
-  <si>
-    <t>SIGN</t>
-  </si>
-  <si>
-    <t>PAID DATE</t>
-  </si>
-  <si>
-    <t>ENGINE</t>
-  </si>
-  <si>
-    <t>GEAR</t>
-  </si>
-  <si>
-    <t>BODY / CABIN</t>
-  </si>
-  <si>
-    <t>TYRES</t>
-  </si>
-  <si>
-    <t>TEST unposted engine work detail</t>
-  </si>
-  <si>
-    <t>TEST unposted gearbox work detail</t>
-  </si>
-  <si>
-    <t>TEST unposted tyres work detail</t>
-  </si>
-  <si>
-    <t>Total Bill</t>
-  </si>
-  <si>
-    <t>TEST unposted body work detail</t>
-  </si>
-  <si>
-    <t>TEST unposted cabin work detail</t>
-  </si>
-  <si>
-    <t>GBT SIGN</t>
-  </si>
-  <si>
-    <t>C.E.O. SIGN</t>
+    <t>Driver signature</t>
+  </si>
+  <si>
+    <t>Driver thumb impression</t>
+  </si>
+  <si>
+    <t>Paid by</t>
+  </si>
+  <si>
+    <t>Authorized signature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signature: __________________
+Name: ____________________
+Date: _____________________</t>
   </si>
   <si>
     <t>Vehicle Advance, Driver Sale, Mobile Load, deductions, tracker and printed settlement totals lack confirmed sources/calculations. Payment and signature spaces remain blank; this is not a finalized payment voucher.</t>
@@ -1066,10 +1059,10 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CF130"/>
+  <dimension ref="A1:CF126"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="84" width="1.9" customWidth="1"/>
+    <col min="1" max="84" width="1.35" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
@@ -2029,7 +2022,7 @@
       <c r="N13" s="5"/>
       <c r="O13" s="5"/>
       <c r="P13" s="7">
-        <v>400</v>
+        <v>250</v>
       </c>
       <c r="Q13" s="7"/>
       <c r="R13" s="7"/>
@@ -2040,7 +2033,7 @@
       <c r="W13" s="7"/>
       <c r="X13" s="7"/>
       <c r="Y13" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z13" s="6"/>
       <c r="AA13" s="6"/>
@@ -2153,7 +2146,7 @@
       <c r="N14" s="5"/>
       <c r="O14" s="5"/>
       <c r="P14" s="7">
-        <v>500</v>
+        <v>150</v>
       </c>
       <c r="Q14" s="7"/>
       <c r="R14" s="7"/>
@@ -2164,7 +2157,7 @@
       <c r="W14" s="7"/>
       <c r="X14" s="7"/>
       <c r="Y14" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z14" s="6"/>
       <c r="AA14" s="6"/>
@@ -2276,19 +2269,19 @@
       <c r="M15" s="5"/>
       <c r="N15" s="5"/>
       <c r="O15" s="5"/>
-      <c r="P15" s="7"/>
+      <c r="P15" s="7">
+        <v>500</v>
+      </c>
       <c r="Q15" s="7"/>
       <c r="R15" s="7"/>
-      <c r="S15" s="7">
-        <v>200</v>
-      </c>
+      <c r="S15" s="7"/>
       <c r="T15" s="7"/>
       <c r="U15" s="7"/>
       <c r="V15" s="7"/>
       <c r="W15" s="7"/>
       <c r="X15" s="7"/>
       <c r="Y15" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z15" s="6"/>
       <c r="AA15" s="6"/>
@@ -2401,7 +2394,7 @@
       <c r="N16" s="5"/>
       <c r="O16" s="5"/>
       <c r="P16" s="7">
-        <v>250</v>
+        <v>400</v>
       </c>
       <c r="Q16" s="7"/>
       <c r="R16" s="7"/>
@@ -2412,7 +2405,7 @@
       <c r="W16" s="7"/>
       <c r="X16" s="7"/>
       <c r="Y16" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z16" s="6"/>
       <c r="AA16" s="6"/>
@@ -2527,16 +2520,16 @@
       <c r="P17" s="7"/>
       <c r="Q17" s="7"/>
       <c r="R17" s="7"/>
-      <c r="S17" s="7"/>
+      <c r="S17" s="7">
+        <v>200</v>
+      </c>
       <c r="T17" s="7"/>
       <c r="U17" s="7"/>
-      <c r="V17" s="7">
-        <v>300</v>
-      </c>
+      <c r="V17" s="7"/>
       <c r="W17" s="7"/>
       <c r="X17" s="7"/>
       <c r="Y17" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z17" s="6"/>
       <c r="AA17" s="6"/>
@@ -2648,19 +2641,19 @@
       <c r="M18" s="5"/>
       <c r="N18" s="5"/>
       <c r="O18" s="5"/>
-      <c r="P18" s="7">
-        <v>150</v>
-      </c>
+      <c r="P18" s="7"/>
       <c r="Q18" s="7"/>
       <c r="R18" s="7"/>
       <c r="S18" s="7"/>
       <c r="T18" s="7"/>
       <c r="U18" s="7"/>
-      <c r="V18" s="7"/>
+      <c r="V18" s="7">
+        <v>300</v>
+      </c>
       <c r="W18" s="7"/>
       <c r="X18" s="7"/>
       <c r="Y18" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z18" s="6"/>
       <c r="AA18" s="6"/>
@@ -2786,7 +2779,7 @@
       <c r="W19" s="12"/>
       <c r="X19" s="12"/>
       <c r="Y19" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z19" s="6"/>
       <c r="AA19" s="6"/>
@@ -2880,7 +2873,7 @@
     </row>
     <row r="20" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y20" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z20" s="6"/>
       <c r="AA20" s="6"/>
@@ -2974,7 +2967,7 @@
     </row>
     <row r="21" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y21" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z21" s="6"/>
       <c r="AA21" s="6"/>
@@ -3068,7 +3061,7 @@
     </row>
     <row r="22" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y22" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z22" s="6"/>
       <c r="AA22" s="6"/>
@@ -3162,7 +3155,7 @@
     </row>
     <row r="23" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y23" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z23" s="6"/>
       <c r="AA23" s="6"/>
@@ -3256,7 +3249,7 @@
     </row>
     <row r="24" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y24" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z24" s="6"/>
       <c r="AA24" s="6"/>
@@ -3350,7 +3343,7 @@
     </row>
     <row r="25" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y25" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z25" s="6"/>
       <c r="AA25" s="6"/>
@@ -3444,7 +3437,7 @@
     </row>
     <row r="26" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y26" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z26" s="6"/>
       <c r="AA26" s="6"/>
@@ -3538,7 +3531,7 @@
     </row>
     <row r="27" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y27" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z27" s="6"/>
       <c r="AA27" s="6"/>
@@ -3632,7 +3625,7 @@
     </row>
     <row r="28" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y28" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z28" s="6"/>
       <c r="AA28" s="6"/>
@@ -3726,7 +3719,7 @@
     </row>
     <row r="29" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y29" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z29" s="6"/>
       <c r="AA29" s="6"/>
@@ -3820,7 +3813,7 @@
     </row>
     <row r="30" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y30" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z30" s="6"/>
       <c r="AA30" s="6"/>
@@ -3914,7 +3907,7 @@
     </row>
     <row r="31" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y31" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z31" s="6"/>
       <c r="AA31" s="6"/>
@@ -4008,7 +4001,7 @@
     </row>
     <row r="32" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y32" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z32" s="6"/>
       <c r="AA32" s="6"/>
@@ -4102,7 +4095,7 @@
     </row>
     <row r="33" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y33" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z33" s="6"/>
       <c r="AA33" s="6"/>
@@ -4196,7 +4189,7 @@
     </row>
     <row r="34" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y34" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z34" s="6"/>
       <c r="AA34" s="6"/>
@@ -4290,7 +4283,7 @@
     </row>
     <row r="35" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y35" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z35" s="6"/>
       <c r="AA35" s="6"/>
@@ -4384,7 +4377,7 @@
     </row>
     <row r="36" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y36" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z36" s="6"/>
       <c r="AA36" s="6"/>
@@ -4478,7 +4471,7 @@
     </row>
     <row r="37" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y37" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z37" s="6"/>
       <c r="AA37" s="6"/>
@@ -4572,7 +4565,7 @@
     </row>
     <row r="38" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y38" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z38" s="6"/>
       <c r="AA38" s="6"/>
@@ -4666,7 +4659,7 @@
     </row>
     <row r="39" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y39" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z39" s="6"/>
       <c r="AA39" s="6"/>
@@ -4760,7 +4753,7 @@
     </row>
     <row r="40" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y40" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z40" s="6"/>
       <c r="AA40" s="6"/>
@@ -4854,7 +4847,7 @@
     </row>
     <row r="41" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y41" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z41" s="6"/>
       <c r="AA41" s="6"/>
@@ -4948,7 +4941,7 @@
     </row>
     <row r="42" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y42" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z42" s="6"/>
       <c r="AA42" s="6"/>
@@ -5042,7 +5035,7 @@
     </row>
     <row r="43" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y43" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z43" s="6"/>
       <c r="AA43" s="6"/>
@@ -5136,7 +5129,7 @@
     </row>
     <row r="44" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y44" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z44" s="6"/>
       <c r="AA44" s="6"/>
@@ -5230,7 +5223,7 @@
     </row>
     <row r="45" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y45" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z45" s="6"/>
       <c r="AA45" s="6"/>
@@ -5324,7 +5317,7 @@
     </row>
     <row r="46" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y46" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z46" s="6"/>
       <c r="AA46" s="6"/>
@@ -5418,7 +5411,7 @@
     </row>
     <row r="47" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y47" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z47" s="6"/>
       <c r="AA47" s="6"/>
@@ -5512,7 +5505,7 @@
     </row>
     <row r="48" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y48" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z48" s="6"/>
       <c r="AA48" s="6"/>
@@ -5606,7 +5599,7 @@
     </row>
     <row r="49" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y49" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z49" s="6"/>
       <c r="AA49" s="6"/>
@@ -5700,7 +5693,7 @@
     </row>
     <row r="50" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y50" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z50" s="6"/>
       <c r="AA50" s="6"/>
@@ -5794,7 +5787,7 @@
     </row>
     <row r="51" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y51" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z51" s="6"/>
       <c r="AA51" s="6"/>
@@ -5888,7 +5881,7 @@
     </row>
     <row r="52" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y52" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z52" s="6"/>
       <c r="AA52" s="6"/>
@@ -5982,7 +5975,7 @@
     </row>
     <row r="53" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y53" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z53" s="6"/>
       <c r="AA53" s="6"/>
@@ -6076,7 +6069,7 @@
     </row>
     <row r="54" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y54" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z54" s="6"/>
       <c r="AA54" s="6"/>
@@ -6170,7 +6163,7 @@
     </row>
     <row r="55" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y55" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z55" s="6"/>
       <c r="AA55" s="6"/>
@@ -6264,7 +6257,7 @@
     </row>
     <row r="56" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y56" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z56" s="6"/>
       <c r="AA56" s="6"/>
@@ -6358,7 +6351,7 @@
     </row>
     <row r="57" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y57" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z57" s="6"/>
       <c r="AA57" s="6"/>
@@ -6452,7 +6445,7 @@
     </row>
     <row r="58" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y58" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z58" s="6"/>
       <c r="AA58" s="6"/>
@@ -6546,7 +6539,7 @@
     </row>
     <row r="59" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y59" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z59" s="6"/>
       <c r="AA59" s="6"/>
@@ -6640,7 +6633,7 @@
     </row>
     <row r="60" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y60" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z60" s="6"/>
       <c r="AA60" s="6"/>
@@ -6734,7 +6727,7 @@
     </row>
     <row r="61" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y61" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z61" s="6"/>
       <c r="AA61" s="6"/>
@@ -6828,7 +6821,7 @@
     </row>
     <row r="62" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y62" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z62" s="6"/>
       <c r="AA62" s="6"/>
@@ -6922,7 +6915,7 @@
     </row>
     <row r="63" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y63" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z63" s="6"/>
       <c r="AA63" s="6"/>
@@ -7016,7 +7009,7 @@
     </row>
     <row r="64" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y64" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z64" s="6"/>
       <c r="AA64" s="6"/>
@@ -7110,7 +7103,7 @@
     </row>
     <row r="65" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y65" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z65" s="6"/>
       <c r="AA65" s="6"/>
@@ -7204,7 +7197,7 @@
     </row>
     <row r="66" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y66" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z66" s="6"/>
       <c r="AA66" s="6"/>
@@ -7298,7 +7291,7 @@
     </row>
     <row r="67" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y67" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z67" s="6"/>
       <c r="AA67" s="6"/>
@@ -7392,7 +7385,7 @@
     </row>
     <row r="68" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y68" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z68" s="6"/>
       <c r="AA68" s="6"/>
@@ -7486,7 +7479,7 @@
     </row>
     <row r="69" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y69" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z69" s="6"/>
       <c r="AA69" s="6"/>
@@ -7580,7 +7573,7 @@
     </row>
     <row r="70" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y70" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z70" s="6"/>
       <c r="AA70" s="6"/>
@@ -7674,7 +7667,7 @@
     </row>
     <row r="71" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y71" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z71" s="6"/>
       <c r="AA71" s="6"/>
@@ -7768,7 +7761,7 @@
     </row>
     <row r="72" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y72" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z72" s="6"/>
       <c r="AA72" s="6"/>
@@ -7862,7 +7855,7 @@
     </row>
     <row r="73" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y73" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z73" s="6"/>
       <c r="AA73" s="6"/>
@@ -7956,7 +7949,7 @@
     </row>
     <row r="74" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y74" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z74" s="6"/>
       <c r="AA74" s="6"/>
@@ -8050,7 +8043,7 @@
     </row>
     <row r="75" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y75" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z75" s="6"/>
       <c r="AA75" s="6"/>
@@ -8144,7 +8137,7 @@
     </row>
     <row r="76" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y76" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z76" s="6"/>
       <c r="AA76" s="6"/>
@@ -8238,7 +8231,7 @@
     </row>
     <row r="77" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y77" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z77" s="6"/>
       <c r="AA77" s="6"/>
@@ -8332,7 +8325,7 @@
     </row>
     <row r="78" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y78" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z78" s="6"/>
       <c r="AA78" s="6"/>
@@ -8426,7 +8419,7 @@
     </row>
     <row r="79" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y79" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z79" s="6"/>
       <c r="AA79" s="6"/>
@@ -8520,7 +8513,7 @@
     </row>
     <row r="80" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y80" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z80" s="6"/>
       <c r="AA80" s="6"/>
@@ -8614,7 +8607,7 @@
     </row>
     <row r="81" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y81" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z81" s="6"/>
       <c r="AA81" s="6"/>
@@ -8708,7 +8701,7 @@
     </row>
     <row r="82" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y82" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z82" s="6"/>
       <c r="AA82" s="6"/>
@@ -8802,7 +8795,7 @@
     </row>
     <row r="83" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y83" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z83" s="6"/>
       <c r="AA83" s="6"/>
@@ -8896,7 +8889,7 @@
     </row>
     <row r="84" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y84" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z84" s="6"/>
       <c r="AA84" s="6"/>
@@ -8990,7 +8983,7 @@
     </row>
     <row r="85" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y85" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z85" s="6"/>
       <c r="AA85" s="6"/>
@@ -9084,7 +9077,7 @@
     </row>
     <row r="86" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y86" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z86" s="6"/>
       <c r="AA86" s="6"/>
@@ -9178,7 +9171,7 @@
     </row>
     <row r="87" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y87" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z87" s="6"/>
       <c r="AA87" s="6"/>
@@ -9272,7 +9265,7 @@
     </row>
     <row r="88" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y88" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z88" s="6"/>
       <c r="AA88" s="6"/>
@@ -9366,7 +9359,7 @@
     </row>
     <row r="89" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y89" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z89" s="6"/>
       <c r="AA89" s="6"/>
@@ -9460,7 +9453,7 @@
     </row>
     <row r="90" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y90" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z90" s="6"/>
       <c r="AA90" s="6"/>
@@ -9554,7 +9547,7 @@
     </row>
     <row r="91" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y91" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z91" s="6"/>
       <c r="AA91" s="6"/>
@@ -9648,7 +9641,7 @@
     </row>
     <row r="92" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y92" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z92" s="6"/>
       <c r="AA92" s="6"/>
@@ -9742,7 +9735,7 @@
     </row>
     <row r="93" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y93" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z93" s="6"/>
       <c r="AA93" s="6"/>
@@ -9836,7 +9829,7 @@
     </row>
     <row r="94" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y94" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z94" s="6"/>
       <c r="AA94" s="6"/>
@@ -9930,7 +9923,7 @@
     </row>
     <row r="95" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y95" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z95" s="6"/>
       <c r="AA95" s="6"/>
@@ -10024,7 +10017,7 @@
     </row>
     <row r="96" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y96" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z96" s="6"/>
       <c r="AA96" s="6"/>
@@ -10118,7 +10111,7 @@
     </row>
     <row r="97" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y97" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z97" s="6"/>
       <c r="AA97" s="6"/>
@@ -10212,7 +10205,7 @@
     </row>
     <row r="98" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y98" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z98" s="6"/>
       <c r="AA98" s="6"/>
@@ -10306,7 +10299,7 @@
     </row>
     <row r="99" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y99" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z99" s="6"/>
       <c r="AA99" s="6"/>
@@ -10400,7 +10393,7 @@
     </row>
     <row r="100" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y100" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z100" s="6"/>
       <c r="AA100" s="6"/>
@@ -10494,7 +10487,7 @@
     </row>
     <row r="101" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y101" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z101" s="6"/>
       <c r="AA101" s="6"/>
@@ -10588,7 +10581,7 @@
     </row>
     <row r="102" ht="26" customHeight="1" spans="25:84" x14ac:dyDescent="0.25">
       <c r="Y102" s="6">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="Z102" s="6"/>
       <c r="AA102" s="6"/>
@@ -10901,7 +10894,7 @@
       <c r="AJ106" s="3"/>
       <c r="AK106" s="3"/>
       <c r="AL106" s="3" t="s">
-        <v>138</v>
+        <v>30</v>
       </c>
       <c r="AM106" s="3"/>
       <c r="AN106" s="3"/>
@@ -10913,7 +10906,7 @@
       <c r="AT106" s="3"/>
       <c r="AU106" s="3"/>
       <c r="AV106" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AW106" s="3"/>
       <c r="AX106" s="3"/>
@@ -10924,7 +10917,7 @@
       <c r="BC106" s="3"/>
       <c r="BD106" s="3"/>
       <c r="BE106" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="BF106" s="3"/>
       <c r="BG106" s="3"/>
@@ -10935,7 +10928,7 @@
       <c r="BL106" s="3"/>
       <c r="BM106" s="3"/>
       <c r="BN106" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="BO106" s="3"/>
       <c r="BP106" s="3"/>
@@ -10947,7 +10940,7 @@
       <c r="BV106" s="3"/>
       <c r="BW106" s="3"/>
       <c r="BX106" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="BY106" s="3"/>
       <c r="BZ106" s="3"/>
@@ -11056,7 +11049,7 @@
     </row>
     <row r="109" ht="22" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B109" s="3"/>
       <c r="C109" s="3"/>
@@ -11144,14 +11137,14 @@
     </row>
     <row r="110" ht="45" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A110" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B110" s="3"/>
       <c r="C110" s="3"/>
       <c r="D110" s="3"/>
       <c r="E110" s="3"/>
       <c r="F110" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G110" s="3"/>
       <c r="H110" s="3"/>
@@ -11159,14 +11152,14 @@
       <c r="J110" s="3"/>
       <c r="K110" s="3"/>
       <c r="L110" s="3" t="s">
-        <v>138</v>
+        <v>30</v>
       </c>
       <c r="M110" s="3"/>
       <c r="N110" s="3"/>
       <c r="O110" s="3"/>
       <c r="P110" s="3"/>
       <c r="Q110" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="R110" s="3"/>
       <c r="S110" s="3"/>
@@ -11180,7 +11173,7 @@
       <c r="Y110" s="3"/>
       <c r="Z110" s="3"/>
       <c r="AA110" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AB110" s="3"/>
       <c r="AC110" s="3"/>
@@ -11188,28 +11181,28 @@
       <c r="AE110" s="3"/>
       <c r="AF110" s="3"/>
       <c r="AG110" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AH110" s="3"/>
       <c r="AI110" s="3"/>
       <c r="AJ110" s="3"/>
       <c r="AK110" s="3"/>
       <c r="AL110" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AM110" s="3"/>
       <c r="AN110" s="3"/>
       <c r="AO110" s="3"/>
       <c r="AP110" s="3"/>
       <c r="AQ110" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AR110" s="3"/>
       <c r="AS110" s="3"/>
       <c r="AT110" s="3"/>
       <c r="AU110" s="3"/>
       <c r="AV110" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="AW110" s="3"/>
       <c r="AX110" s="3"/>
@@ -11217,28 +11210,28 @@
       <c r="AZ110" s="3"/>
       <c r="BA110" s="3"/>
       <c r="BB110" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="BC110" s="3"/>
       <c r="BD110" s="3"/>
       <c r="BE110" s="3"/>
       <c r="BF110" s="3"/>
       <c r="BG110" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="BH110" s="3"/>
       <c r="BI110" s="3"/>
       <c r="BJ110" s="3"/>
       <c r="BK110" s="3"/>
       <c r="BL110" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="BM110" s="3"/>
       <c r="BN110" s="3"/>
       <c r="BO110" s="3"/>
       <c r="BP110" s="3"/>
       <c r="BQ110" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="BR110" s="3"/>
       <c r="BS110" s="3"/>
@@ -11246,14 +11239,14 @@
       <c r="BU110" s="3"/>
       <c r="BV110" s="3"/>
       <c r="BW110" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="BX110" s="3"/>
       <c r="BY110" s="3"/>
       <c r="BZ110" s="3"/>
       <c r="CA110" s="3"/>
       <c r="CB110" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="CC110" s="3"/>
       <c r="CD110" s="3"/>
@@ -11358,7 +11351,7 @@
     </row>
     <row r="113" ht="22" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A113" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
@@ -11380,7 +11373,9 @@
       <c r="S113" s="3"/>
       <c r="T113" s="3"/>
       <c r="U113" s="3"/>
-      <c r="V113" s="3"/>
+      <c r="V113" s="3" t="s">
+        <v>158</v>
+      </c>
       <c r="W113" s="3"/>
       <c r="X113" s="3"/>
       <c r="Y113" s="3"/>
@@ -11401,7 +11396,9 @@
       <c r="AN113" s="3"/>
       <c r="AO113" s="3"/>
       <c r="AP113" s="3"/>
-      <c r="AQ113" s="3"/>
+      <c r="AQ113" s="3" t="s">
+        <v>159</v>
+      </c>
       <c r="AR113" s="3"/>
       <c r="AS113" s="3"/>
       <c r="AT113" s="3"/>
@@ -11422,7 +11419,9 @@
       <c r="BI113" s="3"/>
       <c r="BJ113" s="3"/>
       <c r="BK113" s="3"/>
-      <c r="BL113" s="3"/>
+      <c r="BL113" s="3" t="s">
+        <v>160</v>
+      </c>
       <c r="BM113" s="3"/>
       <c r="BN113" s="3"/>
       <c r="BO113" s="3"/>
@@ -11446,14 +11445,16 @@
     </row>
     <row r="114" ht="45" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A114" s="3" t="s">
-        <v>159</v>
+        <v>16</v>
       </c>
       <c r="B114" s="3"/>
       <c r="C114" s="3"/>
       <c r="D114" s="3"/>
       <c r="E114" s="3"/>
       <c r="F114" s="3"/>
-      <c r="G114" s="3"/>
+      <c r="G114" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="H114" s="3"/>
       <c r="I114" s="3"/>
       <c r="J114" s="3"/>
@@ -11463,47 +11464,53 @@
       <c r="N114" s="3"/>
       <c r="O114" s="3"/>
       <c r="P114" s="3"/>
-      <c r="Q114" s="3"/>
-      <c r="R114" s="3" t="s">
-        <v>160</v>
-      </c>
+      <c r="Q114" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="R114" s="3"/>
       <c r="S114" s="3"/>
       <c r="T114" s="3"/>
       <c r="U114" s="3"/>
-      <c r="V114" s="3"/>
+      <c r="V114" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="W114" s="3"/>
       <c r="X114" s="3"/>
       <c r="Y114" s="3"/>
       <c r="Z114" s="3"/>
       <c r="AA114" s="3"/>
-      <c r="AB114" s="3"/>
+      <c r="AB114" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="AC114" s="3"/>
       <c r="AD114" s="3"/>
       <c r="AE114" s="3"/>
       <c r="AF114" s="3"/>
       <c r="AG114" s="3"/>
       <c r="AH114" s="3"/>
-      <c r="AI114" s="3" t="s">
-        <v>161</v>
-      </c>
+      <c r="AI114" s="3"/>
       <c r="AJ114" s="3"/>
       <c r="AK114" s="3"/>
-      <c r="AL114" s="3"/>
+      <c r="AL114" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="AM114" s="3"/>
       <c r="AN114" s="3"/>
       <c r="AO114" s="3"/>
       <c r="AP114" s="3"/>
-      <c r="AQ114" s="3"/>
+      <c r="AQ114" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="AR114" s="3"/>
       <c r="AS114" s="3"/>
       <c r="AT114" s="3"/>
       <c r="AU114" s="3"/>
       <c r="AV114" s="3"/>
-      <c r="AW114" s="3"/>
+      <c r="AW114" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="AX114" s="3"/>
-      <c r="AY114" s="3" t="s">
-        <v>162</v>
-      </c>
+      <c r="AY114" s="3"/>
       <c r="AZ114" s="3"/>
       <c r="BA114" s="3"/>
       <c r="BB114" s="3"/>
@@ -11511,20 +11518,24 @@
       <c r="BD114" s="3"/>
       <c r="BE114" s="3"/>
       <c r="BF114" s="3"/>
-      <c r="BG114" s="3"/>
+      <c r="BG114" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="BH114" s="3"/>
       <c r="BI114" s="3"/>
       <c r="BJ114" s="3"/>
       <c r="BK114" s="3"/>
-      <c r="BL114" s="3"/>
+      <c r="BL114" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="BM114" s="3"/>
       <c r="BN114" s="3"/>
       <c r="BO114" s="3"/>
-      <c r="BP114" s="3" t="s">
-        <v>163</v>
-      </c>
+      <c r="BP114" s="3"/>
       <c r="BQ114" s="3"/>
-      <c r="BR114" s="3"/>
+      <c r="BR114" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="BS114" s="3"/>
       <c r="BT114" s="3"/>
       <c r="BU114" s="3"/>
@@ -11534,20 +11545,26 @@
       <c r="BY114" s="3"/>
       <c r="BZ114" s="3"/>
       <c r="CA114" s="3"/>
-      <c r="CB114" s="3"/>
+      <c r="CB114" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="CC114" s="3"/>
       <c r="CD114" s="3"/>
       <c r="CE114" s="3"/>
       <c r="CF114" s="3"/>
     </row>
-    <row r="115" ht="42" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A115" s="5"/>
-      <c r="B115" s="5"/>
-      <c r="C115" s="5"/>
-      <c r="D115" s="5"/>
-      <c r="E115" s="5"/>
-      <c r="F115" s="5"/>
-      <c r="G115" s="5"/>
+    <row r="115" ht="26" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
+      <c r="A115" s="6">
+        <v>46023</v>
+      </c>
+      <c r="B115" s="6"/>
+      <c r="C115" s="6"/>
+      <c r="D115" s="6"/>
+      <c r="E115" s="6"/>
+      <c r="F115" s="6"/>
+      <c r="G115" s="5" t="s">
+        <v>40</v>
+      </c>
       <c r="H115" s="5"/>
       <c r="I115" s="5"/>
       <c r="J115" s="5"/>
@@ -11557,18 +11574,24 @@
       <c r="N115" s="5"/>
       <c r="O115" s="5"/>
       <c r="P115" s="5"/>
-      <c r="Q115" s="5"/>
-      <c r="R115" s="5"/>
-      <c r="S115" s="5"/>
-      <c r="T115" s="5"/>
-      <c r="U115" s="5"/>
-      <c r="V115" s="5"/>
-      <c r="W115" s="5"/>
-      <c r="X115" s="5"/>
-      <c r="Y115" s="5"/>
-      <c r="Z115" s="5"/>
-      <c r="AA115" s="5"/>
-      <c r="AB115" s="5"/>
+      <c r="Q115" s="7">
+        <v>500</v>
+      </c>
+      <c r="R115" s="7"/>
+      <c r="S115" s="7"/>
+      <c r="T115" s="7"/>
+      <c r="U115" s="7"/>
+      <c r="V115" s="6">
+        <v>46023</v>
+      </c>
+      <c r="W115" s="6"/>
+      <c r="X115" s="6"/>
+      <c r="Y115" s="6"/>
+      <c r="Z115" s="6"/>
+      <c r="AA115" s="6"/>
+      <c r="AB115" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="AC115" s="5"/>
       <c r="AD115" s="5"/>
       <c r="AE115" s="5"/>
@@ -11578,18 +11601,24 @@
       <c r="AI115" s="5"/>
       <c r="AJ115" s="5"/>
       <c r="AK115" s="5"/>
-      <c r="AL115" s="5"/>
-      <c r="AM115" s="5"/>
-      <c r="AN115" s="5"/>
-      <c r="AO115" s="5"/>
-      <c r="AP115" s="5"/>
-      <c r="AQ115" s="5"/>
-      <c r="AR115" s="5"/>
-      <c r="AS115" s="5"/>
-      <c r="AT115" s="5"/>
-      <c r="AU115" s="5"/>
-      <c r="AV115" s="5"/>
-      <c r="AW115" s="5"/>
+      <c r="AL115" s="7">
+        <v>250</v>
+      </c>
+      <c r="AM115" s="7"/>
+      <c r="AN115" s="7"/>
+      <c r="AO115" s="7"/>
+      <c r="AP115" s="7"/>
+      <c r="AQ115" s="6">
+        <v>46023</v>
+      </c>
+      <c r="AR115" s="6"/>
+      <c r="AS115" s="6"/>
+      <c r="AT115" s="6"/>
+      <c r="AU115" s="6"/>
+      <c r="AV115" s="6"/>
+      <c r="AW115" s="5" t="s">
+        <v>38</v>
+      </c>
       <c r="AX115" s="5"/>
       <c r="AY115" s="5"/>
       <c r="AZ115" s="5"/>
@@ -11599,1039 +11628,745 @@
       <c r="BD115" s="5"/>
       <c r="BE115" s="5"/>
       <c r="BF115" s="5"/>
-      <c r="BG115" s="5"/>
-      <c r="BH115" s="5"/>
-      <c r="BI115" s="5"/>
-      <c r="BJ115" s="5"/>
-      <c r="BK115" s="5"/>
-      <c r="BL115" s="5"/>
-      <c r="BM115" s="5"/>
-      <c r="BN115" s="5"/>
-      <c r="BO115" s="5"/>
+      <c r="BG115" s="7">
+        <v>150</v>
+      </c>
+      <c r="BH115" s="7"/>
+      <c r="BI115" s="7"/>
+      <c r="BJ115" s="7"/>
+      <c r="BK115" s="7"/>
+      <c r="BL115" s="6">
+        <v>46023</v>
+      </c>
+      <c r="BM115" s="6"/>
+      <c r="BN115" s="6"/>
+      <c r="BO115" s="6"/>
       <c r="BP115" s="6"/>
       <c r="BQ115" s="6"/>
-      <c r="BR115" s="6"/>
-      <c r="BS115" s="6"/>
-      <c r="BT115" s="6"/>
-      <c r="BU115" s="6"/>
-      <c r="BV115" s="6"/>
-      <c r="BW115" s="6"/>
-      <c r="BX115" s="6"/>
-      <c r="BY115" s="6"/>
-      <c r="BZ115" s="6"/>
-      <c r="CA115" s="6"/>
-      <c r="CB115" s="6"/>
-      <c r="CC115" s="6"/>
-      <c r="CD115" s="6"/>
-      <c r="CE115" s="6"/>
-      <c r="CF115" s="6"/>
+      <c r="BR115" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="BS115" s="5"/>
+      <c r="BT115" s="5"/>
+      <c r="BU115" s="5"/>
+      <c r="BV115" s="5"/>
+      <c r="BW115" s="5"/>
+      <c r="BX115" s="5"/>
+      <c r="BY115" s="5"/>
+      <c r="BZ115" s="5"/>
+      <c r="CA115" s="5"/>
+      <c r="CB115" s="7">
+        <v>300</v>
+      </c>
+      <c r="CC115" s="7"/>
+      <c r="CD115" s="7"/>
+      <c r="CE115" s="7"/>
+      <c r="CF115" s="7"/>
     </row>
-    <row r="117" ht="22" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A117" s="3" t="s">
+    <row r="116" ht="26" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
+      <c r="A116" s="6"/>
+      <c r="B116" s="6"/>
+      <c r="C116" s="6"/>
+      <c r="D116" s="6"/>
+      <c r="E116" s="6"/>
+      <c r="F116" s="6"/>
+      <c r="G116" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="H116" s="5"/>
+      <c r="I116" s="5"/>
+      <c r="J116" s="5"/>
+      <c r="K116" s="5"/>
+      <c r="L116" s="5"/>
+      <c r="M116" s="5"/>
+      <c r="N116" s="5"/>
+      <c r="O116" s="5"/>
+      <c r="P116" s="5"/>
+      <c r="Q116" s="7"/>
+      <c r="R116" s="7"/>
+      <c r="S116" s="7"/>
+      <c r="T116" s="7"/>
+      <c r="U116" s="7"/>
+      <c r="V116" s="6"/>
+      <c r="W116" s="6"/>
+      <c r="X116" s="6"/>
+      <c r="Y116" s="6"/>
+      <c r="Z116" s="6"/>
+      <c r="AA116" s="6"/>
+      <c r="AB116" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="AC116" s="5"/>
+      <c r="AD116" s="5"/>
+      <c r="AE116" s="5"/>
+      <c r="AF116" s="5"/>
+      <c r="AG116" s="5"/>
+      <c r="AH116" s="5"/>
+      <c r="AI116" s="5"/>
+      <c r="AJ116" s="5"/>
+      <c r="AK116" s="5"/>
+      <c r="AL116" s="7"/>
+      <c r="AM116" s="7"/>
+      <c r="AN116" s="7"/>
+      <c r="AO116" s="7"/>
+      <c r="AP116" s="7"/>
+      <c r="AQ116" s="6">
+        <v>46023</v>
+      </c>
+      <c r="AR116" s="6"/>
+      <c r="AS116" s="6"/>
+      <c r="AT116" s="6"/>
+      <c r="AU116" s="6"/>
+      <c r="AV116" s="6"/>
+      <c r="AW116" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AX116" s="5"/>
+      <c r="AY116" s="5"/>
+      <c r="AZ116" s="5"/>
+      <c r="BA116" s="5"/>
+      <c r="BB116" s="5"/>
+      <c r="BC116" s="5"/>
+      <c r="BD116" s="5"/>
+      <c r="BE116" s="5"/>
+      <c r="BF116" s="5"/>
+      <c r="BG116" s="7">
+        <v>400</v>
+      </c>
+      <c r="BH116" s="7"/>
+      <c r="BI116" s="7"/>
+      <c r="BJ116" s="7"/>
+      <c r="BK116" s="7"/>
+      <c r="BL116" s="6"/>
+      <c r="BM116" s="6"/>
+      <c r="BN116" s="6"/>
+      <c r="BO116" s="6"/>
+      <c r="BP116" s="6"/>
+      <c r="BQ116" s="6"/>
+      <c r="BR116" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="BS116" s="5"/>
+      <c r="BT116" s="5"/>
+      <c r="BU116" s="5"/>
+      <c r="BV116" s="5"/>
+      <c r="BW116" s="5"/>
+      <c r="BX116" s="5"/>
+      <c r="BY116" s="5"/>
+      <c r="BZ116" s="5"/>
+      <c r="CA116" s="5"/>
+      <c r="CB116" s="7"/>
+      <c r="CC116" s="7"/>
+      <c r="CD116" s="7"/>
+      <c r="CE116" s="7"/>
+      <c r="CF116" s="7"/>
+    </row>
+    <row r="117" ht="26" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
+      <c r="A117" s="10"/>
+      <c r="B117" s="10"/>
+      <c r="C117" s="10"/>
+      <c r="D117" s="10"/>
+      <c r="E117" s="10"/>
+      <c r="F117" s="10"/>
+      <c r="G117" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="B117" s="3"/>
-      <c r="C117" s="3"/>
-      <c r="D117" s="3"/>
-      <c r="E117" s="3"/>
-      <c r="F117" s="3"/>
-      <c r="G117" s="3"/>
-      <c r="H117" s="3"/>
-      <c r="I117" s="3"/>
-      <c r="J117" s="3"/>
-      <c r="K117" s="3"/>
-      <c r="L117" s="3"/>
-      <c r="M117" s="3"/>
-      <c r="N117" s="3"/>
-      <c r="O117" s="3"/>
-      <c r="P117" s="3"/>
-      <c r="Q117" s="3"/>
-      <c r="R117" s="3"/>
-      <c r="S117" s="3"/>
-      <c r="T117" s="3"/>
-      <c r="U117" s="3"/>
-      <c r="V117" s="3" t="s">
+      <c r="H117" s="11"/>
+      <c r="I117" s="11"/>
+      <c r="J117" s="11"/>
+      <c r="K117" s="11"/>
+      <c r="L117" s="11"/>
+      <c r="M117" s="11"/>
+      <c r="N117" s="11"/>
+      <c r="O117" s="11"/>
+      <c r="P117" s="11"/>
+      <c r="Q117" s="12">
+        <v>500</v>
+      </c>
+      <c r="R117" s="12"/>
+      <c r="S117" s="12"/>
+      <c r="T117" s="12"/>
+      <c r="U117" s="12"/>
+      <c r="V117" s="10"/>
+      <c r="W117" s="10"/>
+      <c r="X117" s="10"/>
+      <c r="Y117" s="10"/>
+      <c r="Z117" s="10"/>
+      <c r="AA117" s="10"/>
+      <c r="AB117" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="AC117" s="11"/>
+      <c r="AD117" s="11"/>
+      <c r="AE117" s="11"/>
+      <c r="AF117" s="11"/>
+      <c r="AG117" s="11"/>
+      <c r="AH117" s="11"/>
+      <c r="AI117" s="11"/>
+      <c r="AJ117" s="11"/>
+      <c r="AK117" s="11"/>
+      <c r="AL117" s="12">
+        <v>250</v>
+      </c>
+      <c r="AM117" s="12"/>
+      <c r="AN117" s="12"/>
+      <c r="AO117" s="12"/>
+      <c r="AP117" s="12"/>
+      <c r="AQ117" s="6"/>
+      <c r="AR117" s="6"/>
+      <c r="AS117" s="6"/>
+      <c r="AT117" s="6"/>
+      <c r="AU117" s="6"/>
+      <c r="AV117" s="6"/>
+      <c r="AW117" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="W117" s="3"/>
-      <c r="X117" s="3"/>
-      <c r="Y117" s="3"/>
-      <c r="Z117" s="3"/>
-      <c r="AA117" s="3"/>
-      <c r="AB117" s="3"/>
-      <c r="AC117" s="3"/>
-      <c r="AD117" s="3"/>
-      <c r="AE117" s="3"/>
-      <c r="AF117" s="3"/>
-      <c r="AG117" s="3"/>
-      <c r="AH117" s="3"/>
-      <c r="AI117" s="3"/>
-      <c r="AJ117" s="3"/>
-      <c r="AK117" s="3"/>
-      <c r="AL117" s="3"/>
-      <c r="AM117" s="3"/>
-      <c r="AN117" s="3"/>
-      <c r="AO117" s="3"/>
-      <c r="AP117" s="3"/>
-      <c r="AQ117" s="3" t="s">
+      <c r="AX117" s="5"/>
+      <c r="AY117" s="5"/>
+      <c r="AZ117" s="5"/>
+      <c r="BA117" s="5"/>
+      <c r="BB117" s="5"/>
+      <c r="BC117" s="5"/>
+      <c r="BD117" s="5"/>
+      <c r="BE117" s="5"/>
+      <c r="BF117" s="5"/>
+      <c r="BG117" s="7"/>
+      <c r="BH117" s="7"/>
+      <c r="BI117" s="7"/>
+      <c r="BJ117" s="7"/>
+      <c r="BK117" s="7"/>
+      <c r="BL117" s="10"/>
+      <c r="BM117" s="10"/>
+      <c r="BN117" s="10"/>
+      <c r="BO117" s="10"/>
+      <c r="BP117" s="10"/>
+      <c r="BQ117" s="10"/>
+      <c r="BR117" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="BS117" s="11"/>
+      <c r="BT117" s="11"/>
+      <c r="BU117" s="11"/>
+      <c r="BV117" s="11"/>
+      <c r="BW117" s="11"/>
+      <c r="BX117" s="11"/>
+      <c r="BY117" s="11"/>
+      <c r="BZ117" s="11"/>
+      <c r="CA117" s="11"/>
+      <c r="CB117" s="12">
+        <v>300</v>
+      </c>
+      <c r="CC117" s="12"/>
+      <c r="CD117" s="12"/>
+      <c r="CE117" s="12"/>
+      <c r="CF117" s="12"/>
+    </row>
+    <row r="118" ht="26" customHeight="1" spans="43:63" x14ac:dyDescent="0.25">
+      <c r="AQ118" s="6"/>
+      <c r="AR118" s="6"/>
+      <c r="AS118" s="6"/>
+      <c r="AT118" s="6"/>
+      <c r="AU118" s="6"/>
+      <c r="AV118" s="6"/>
+      <c r="AW118" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="AR117" s="3"/>
-      <c r="AS117" s="3"/>
-      <c r="AT117" s="3"/>
-      <c r="AU117" s="3"/>
-      <c r="AV117" s="3"/>
-      <c r="AW117" s="3"/>
-      <c r="AX117" s="3"/>
-      <c r="AY117" s="3"/>
-      <c r="AZ117" s="3"/>
-      <c r="BA117" s="3"/>
-      <c r="BB117" s="3"/>
-      <c r="BC117" s="3"/>
-      <c r="BD117" s="3"/>
-      <c r="BE117" s="3"/>
-      <c r="BF117" s="3"/>
-      <c r="BG117" s="3"/>
-      <c r="BH117" s="3"/>
-      <c r="BI117" s="3"/>
-      <c r="BJ117" s="3"/>
-      <c r="BK117" s="3"/>
-      <c r="BL117" s="3" t="s">
+      <c r="AX118" s="5"/>
+      <c r="AY118" s="5"/>
+      <c r="AZ118" s="5"/>
+      <c r="BA118" s="5"/>
+      <c r="BB118" s="5"/>
+      <c r="BC118" s="5"/>
+      <c r="BD118" s="5"/>
+      <c r="BE118" s="5"/>
+      <c r="BF118" s="5"/>
+      <c r="BG118" s="7"/>
+      <c r="BH118" s="7"/>
+      <c r="BI118" s="7"/>
+      <c r="BJ118" s="7"/>
+      <c r="BK118" s="7"/>
+    </row>
+    <row r="119" ht="24" customHeight="1" spans="43:63" x14ac:dyDescent="0.25">
+      <c r="AQ119" s="10"/>
+      <c r="AR119" s="10"/>
+      <c r="AS119" s="10"/>
+      <c r="AT119" s="10"/>
+      <c r="AU119" s="10"/>
+      <c r="AV119" s="10"/>
+      <c r="AW119" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="AX119" s="11"/>
+      <c r="AY119" s="11"/>
+      <c r="AZ119" s="11"/>
+      <c r="BA119" s="11"/>
+      <c r="BB119" s="11"/>
+      <c r="BC119" s="11"/>
+      <c r="BD119" s="11"/>
+      <c r="BE119" s="11"/>
+      <c r="BF119" s="11"/>
+      <c r="BG119" s="12">
+        <v>550</v>
+      </c>
+      <c r="BH119" s="12"/>
+      <c r="BI119" s="12"/>
+      <c r="BJ119" s="12"/>
+      <c r="BK119" s="12"/>
+    </row>
+    <row r="121" ht="22" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
+      <c r="A121" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="BM117" s="3"/>
-      <c r="BN117" s="3"/>
-      <c r="BO117" s="3"/>
-      <c r="BP117" s="3"/>
-      <c r="BQ117" s="3"/>
-      <c r="BR117" s="3"/>
-      <c r="BS117" s="3"/>
-      <c r="BT117" s="3"/>
-      <c r="BU117" s="3"/>
-      <c r="BV117" s="3"/>
-      <c r="BW117" s="3"/>
-      <c r="BX117" s="3"/>
-      <c r="BY117" s="3"/>
-      <c r="BZ117" s="3"/>
-      <c r="CA117" s="3"/>
-      <c r="CB117" s="3"/>
-      <c r="CC117" s="3"/>
-      <c r="CD117" s="3"/>
-      <c r="CE117" s="3"/>
-      <c r="CF117" s="3"/>
+      <c r="B121" s="3"/>
+      <c r="C121" s="3"/>
+      <c r="D121" s="3"/>
+      <c r="E121" s="3"/>
+      <c r="F121" s="3"/>
+      <c r="G121" s="3"/>
+      <c r="H121" s="3"/>
+      <c r="I121" s="3"/>
+      <c r="J121" s="3"/>
+      <c r="K121" s="3"/>
+      <c r="L121" s="3"/>
+      <c r="M121" s="3"/>
+      <c r="N121" s="3"/>
+      <c r="O121" s="3"/>
+      <c r="P121" s="3"/>
+      <c r="Q121" s="3"/>
+      <c r="R121" s="3"/>
+      <c r="S121" s="3"/>
+      <c r="T121" s="3"/>
+      <c r="U121" s="3"/>
+      <c r="V121" s="3"/>
+      <c r="W121" s="3"/>
+      <c r="X121" s="3"/>
+      <c r="Y121" s="3"/>
+      <c r="Z121" s="3"/>
+      <c r="AA121" s="3"/>
+      <c r="AB121" s="3"/>
+      <c r="AC121" s="3"/>
+      <c r="AD121" s="3"/>
+      <c r="AE121" s="3"/>
+      <c r="AF121" s="3"/>
+      <c r="AG121" s="3"/>
+      <c r="AH121" s="3"/>
+      <c r="AI121" s="3"/>
+      <c r="AJ121" s="3"/>
+      <c r="AK121" s="3"/>
+      <c r="AL121" s="3"/>
+      <c r="AM121" s="3"/>
+      <c r="AN121" s="3"/>
+      <c r="AO121" s="3"/>
+      <c r="AP121" s="3"/>
+      <c r="AQ121" s="3"/>
+      <c r="AR121" s="3"/>
+      <c r="AS121" s="3"/>
+      <c r="AT121" s="3"/>
+      <c r="AU121" s="3"/>
+      <c r="AV121" s="3"/>
+      <c r="AW121" s="3"/>
+      <c r="AX121" s="3"/>
+      <c r="AY121" s="3"/>
+      <c r="AZ121" s="3"/>
+      <c r="BA121" s="3"/>
+      <c r="BB121" s="3"/>
+      <c r="BC121" s="3"/>
+      <c r="BD121" s="3"/>
+      <c r="BE121" s="3"/>
+      <c r="BF121" s="3"/>
+      <c r="BG121" s="3"/>
+      <c r="BH121" s="3"/>
+      <c r="BI121" s="3"/>
+      <c r="BJ121" s="3"/>
+      <c r="BK121" s="3"/>
+      <c r="BL121" s="3"/>
+      <c r="BM121" s="3"/>
+      <c r="BN121" s="3"/>
+      <c r="BO121" s="3"/>
+      <c r="BP121" s="3"/>
+      <c r="BQ121" s="3"/>
+      <c r="BR121" s="3"/>
+      <c r="BS121" s="3"/>
+      <c r="BT121" s="3"/>
+      <c r="BU121" s="3"/>
+      <c r="BV121" s="3"/>
+      <c r="BW121" s="3"/>
+      <c r="BX121" s="3"/>
+      <c r="BY121" s="3"/>
+      <c r="BZ121" s="3"/>
+      <c r="CA121" s="3"/>
+      <c r="CB121" s="3"/>
+      <c r="CC121" s="3"/>
+      <c r="CD121" s="3"/>
+      <c r="CE121" s="3"/>
+      <c r="CF121" s="3"/>
     </row>
-    <row r="118" ht="45" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A118" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B118" s="3"/>
-      <c r="C118" s="3"/>
-      <c r="D118" s="3"/>
-      <c r="E118" s="3"/>
-      <c r="F118" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G118" s="3"/>
-      <c r="H118" s="3"/>
-      <c r="I118" s="3"/>
-      <c r="J118" s="3"/>
-      <c r="K118" s="3"/>
-      <c r="L118" s="3"/>
-      <c r="M118" s="3"/>
-      <c r="N118" s="3"/>
-      <c r="O118" s="3"/>
-      <c r="P118" s="3"/>
-      <c r="Q118" s="3"/>
-      <c r="R118" s="3"/>
-      <c r="S118" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="T118" s="3"/>
-      <c r="U118" s="3"/>
-      <c r="V118" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="W118" s="3"/>
-      <c r="X118" s="3"/>
-      <c r="Y118" s="3"/>
-      <c r="Z118" s="3"/>
-      <c r="AA118" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="AB118" s="3"/>
-      <c r="AC118" s="3"/>
-      <c r="AD118" s="3"/>
-      <c r="AE118" s="3"/>
-      <c r="AF118" s="3"/>
-      <c r="AG118" s="3"/>
-      <c r="AH118" s="3"/>
-      <c r="AI118" s="3"/>
-      <c r="AJ118" s="3"/>
-      <c r="AK118" s="3"/>
-      <c r="AL118" s="3"/>
-      <c r="AM118" s="3"/>
-      <c r="AN118" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="AO118" s="3"/>
-      <c r="AP118" s="3"/>
-      <c r="AQ118" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="AR118" s="3"/>
-      <c r="AS118" s="3"/>
-      <c r="AT118" s="3"/>
-      <c r="AU118" s="3"/>
-      <c r="AV118" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="AW118" s="3"/>
-      <c r="AX118" s="3"/>
-      <c r="AY118" s="3"/>
-      <c r="AZ118" s="3"/>
-      <c r="BA118" s="3"/>
-      <c r="BB118" s="3"/>
-      <c r="BC118" s="3"/>
-      <c r="BD118" s="3"/>
-      <c r="BE118" s="3"/>
-      <c r="BF118" s="3"/>
-      <c r="BG118" s="3"/>
-      <c r="BH118" s="3"/>
-      <c r="BI118" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="BJ118" s="3"/>
-      <c r="BK118" s="3"/>
-      <c r="BL118" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="BM118" s="3"/>
-      <c r="BN118" s="3"/>
-      <c r="BO118" s="3"/>
-      <c r="BP118" s="3"/>
-      <c r="BQ118" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="BR118" s="3"/>
-      <c r="BS118" s="3"/>
-      <c r="BT118" s="3"/>
-      <c r="BU118" s="3"/>
-      <c r="BV118" s="3"/>
-      <c r="BW118" s="3"/>
-      <c r="BX118" s="3"/>
-      <c r="BY118" s="3"/>
-      <c r="BZ118" s="3"/>
-      <c r="CA118" s="3"/>
-      <c r="CB118" s="3"/>
-      <c r="CC118" s="3"/>
-      <c r="CD118" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="CE118" s="3"/>
-      <c r="CF118" s="3"/>
+    <row r="122" ht="45" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
+      <c r="A122" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B122" s="3"/>
+      <c r="C122" s="3"/>
+      <c r="D122" s="3"/>
+      <c r="E122" s="3"/>
+      <c r="F122" s="3"/>
+      <c r="G122" s="3"/>
+      <c r="H122" s="3"/>
+      <c r="I122" s="3"/>
+      <c r="J122" s="3"/>
+      <c r="K122" s="3"/>
+      <c r="L122" s="3"/>
+      <c r="M122" s="3"/>
+      <c r="N122" s="3"/>
+      <c r="O122" s="3"/>
+      <c r="P122" s="3"/>
+      <c r="Q122" s="3"/>
+      <c r="R122" s="3"/>
+      <c r="S122" s="3"/>
+      <c r="T122" s="3"/>
+      <c r="U122" s="3"/>
+      <c r="V122" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="W122" s="3"/>
+      <c r="X122" s="3"/>
+      <c r="Y122" s="3"/>
+      <c r="Z122" s="3"/>
+      <c r="AA122" s="3"/>
+      <c r="AB122" s="3"/>
+      <c r="AC122" s="3"/>
+      <c r="AD122" s="3"/>
+      <c r="AE122" s="3"/>
+      <c r="AF122" s="3"/>
+      <c r="AG122" s="3"/>
+      <c r="AH122" s="3"/>
+      <c r="AI122" s="3"/>
+      <c r="AJ122" s="3"/>
+      <c r="AK122" s="3"/>
+      <c r="AL122" s="3"/>
+      <c r="AM122" s="3"/>
+      <c r="AN122" s="3"/>
+      <c r="AO122" s="3"/>
+      <c r="AP122" s="3"/>
+      <c r="AQ122" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="AR122" s="3"/>
+      <c r="AS122" s="3"/>
+      <c r="AT122" s="3"/>
+      <c r="AU122" s="3"/>
+      <c r="AV122" s="3"/>
+      <c r="AW122" s="3"/>
+      <c r="AX122" s="3"/>
+      <c r="AY122" s="3"/>
+      <c r="AZ122" s="3"/>
+      <c r="BA122" s="3"/>
+      <c r="BB122" s="3"/>
+      <c r="BC122" s="3"/>
+      <c r="BD122" s="3"/>
+      <c r="BE122" s="3"/>
+      <c r="BF122" s="3"/>
+      <c r="BG122" s="3"/>
+      <c r="BH122" s="3"/>
+      <c r="BI122" s="3"/>
+      <c r="BJ122" s="3"/>
+      <c r="BK122" s="3"/>
+      <c r="BL122" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="BM122" s="3"/>
+      <c r="BN122" s="3"/>
+      <c r="BO122" s="3"/>
+      <c r="BP122" s="3"/>
+      <c r="BQ122" s="3"/>
+      <c r="BR122" s="3"/>
+      <c r="BS122" s="3"/>
+      <c r="BT122" s="3"/>
+      <c r="BU122" s="3"/>
+      <c r="BV122" s="3"/>
+      <c r="BW122" s="3"/>
+      <c r="BX122" s="3"/>
+      <c r="BY122" s="3"/>
+      <c r="BZ122" s="3"/>
+      <c r="CA122" s="3"/>
+      <c r="CB122" s="3"/>
+      <c r="CC122" s="3"/>
+      <c r="CD122" s="3"/>
+      <c r="CE122" s="3"/>
+      <c r="CF122" s="3"/>
     </row>
-    <row r="119" ht="26" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A119" s="6">
-        <v>46023</v>
-      </c>
-      <c r="B119" s="6"/>
-      <c r="C119" s="6"/>
-      <c r="D119" s="6"/>
-      <c r="E119" s="6"/>
-      <c r="F119" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="G119" s="5"/>
-      <c r="H119" s="5"/>
-      <c r="I119" s="5"/>
-      <c r="J119" s="5"/>
-      <c r="K119" s="5"/>
-      <c r="L119" s="5"/>
-      <c r="M119" s="5"/>
-      <c r="N119" s="5"/>
-      <c r="O119" s="5"/>
-      <c r="P119" s="5"/>
-      <c r="Q119" s="5"/>
-      <c r="R119" s="5"/>
-      <c r="S119" s="7">
-        <v>500</v>
-      </c>
-      <c r="T119" s="7"/>
-      <c r="U119" s="7"/>
-      <c r="V119" s="6">
-        <v>46023</v>
-      </c>
-      <c r="W119" s="6"/>
-      <c r="X119" s="6"/>
-      <c r="Y119" s="6"/>
-      <c r="Z119" s="6"/>
-      <c r="AA119" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="AB119" s="5"/>
-      <c r="AC119" s="5"/>
-      <c r="AD119" s="5"/>
-      <c r="AE119" s="5"/>
-      <c r="AF119" s="5"/>
-      <c r="AG119" s="5"/>
-      <c r="AH119" s="5"/>
-      <c r="AI119" s="5"/>
-      <c r="AJ119" s="5"/>
-      <c r="AK119" s="5"/>
-      <c r="AL119" s="5"/>
-      <c r="AM119" s="5"/>
-      <c r="AN119" s="7">
-        <v>250</v>
-      </c>
-      <c r="AO119" s="7"/>
-      <c r="AP119" s="7"/>
-      <c r="AQ119" s="6">
-        <v>46023</v>
-      </c>
-      <c r="AR119" s="6"/>
-      <c r="AS119" s="6"/>
-      <c r="AT119" s="6"/>
-      <c r="AU119" s="6"/>
-      <c r="AV119" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="AW119" s="5"/>
-      <c r="AX119" s="5"/>
-      <c r="AY119" s="5"/>
-      <c r="AZ119" s="5"/>
-      <c r="BA119" s="5"/>
-      <c r="BB119" s="5"/>
-      <c r="BC119" s="5"/>
-      <c r="BD119" s="5"/>
-      <c r="BE119" s="5"/>
-      <c r="BF119" s="5"/>
-      <c r="BG119" s="5"/>
-      <c r="BH119" s="5"/>
-      <c r="BI119" s="7">
-        <v>400</v>
-      </c>
-      <c r="BJ119" s="7"/>
-      <c r="BK119" s="7"/>
-      <c r="BL119" s="6">
-        <v>46023</v>
-      </c>
-      <c r="BM119" s="6"/>
-      <c r="BN119" s="6"/>
-      <c r="BO119" s="6"/>
-      <c r="BP119" s="6"/>
-      <c r="BQ119" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="BR119" s="5"/>
-      <c r="BS119" s="5"/>
-      <c r="BT119" s="5"/>
-      <c r="BU119" s="5"/>
-      <c r="BV119" s="5"/>
-      <c r="BW119" s="5"/>
-      <c r="BX119" s="5"/>
-      <c r="BY119" s="5"/>
-      <c r="BZ119" s="5"/>
-      <c r="CA119" s="5"/>
-      <c r="CB119" s="5"/>
-      <c r="CC119" s="5"/>
-      <c r="CD119" s="7">
-        <v>300</v>
-      </c>
-      <c r="CE119" s="7"/>
-      <c r="CF119" s="7"/>
+    <row r="123" ht="85" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
+      <c r="A123" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B123" s="5"/>
+      <c r="C123" s="5"/>
+      <c r="D123" s="5"/>
+      <c r="E123" s="5"/>
+      <c r="F123" s="5"/>
+      <c r="G123" s="5"/>
+      <c r="H123" s="5"/>
+      <c r="I123" s="5"/>
+      <c r="J123" s="5"/>
+      <c r="K123" s="5"/>
+      <c r="L123" s="5"/>
+      <c r="M123" s="5"/>
+      <c r="N123" s="5"/>
+      <c r="O123" s="5"/>
+      <c r="P123" s="5"/>
+      <c r="Q123" s="5"/>
+      <c r="R123" s="5"/>
+      <c r="S123" s="5"/>
+      <c r="T123" s="5"/>
+      <c r="U123" s="5"/>
+      <c r="V123" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="W123" s="5"/>
+      <c r="X123" s="5"/>
+      <c r="Y123" s="5"/>
+      <c r="Z123" s="5"/>
+      <c r="AA123" s="5"/>
+      <c r="AB123" s="5"/>
+      <c r="AC123" s="5"/>
+      <c r="AD123" s="5"/>
+      <c r="AE123" s="5"/>
+      <c r="AF123" s="5"/>
+      <c r="AG123" s="5"/>
+      <c r="AH123" s="5"/>
+      <c r="AI123" s="5"/>
+      <c r="AJ123" s="5"/>
+      <c r="AK123" s="5"/>
+      <c r="AL123" s="5"/>
+      <c r="AM123" s="5"/>
+      <c r="AN123" s="5"/>
+      <c r="AO123" s="5"/>
+      <c r="AP123" s="5"/>
+      <c r="AQ123" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="AR123" s="5"/>
+      <c r="AS123" s="5"/>
+      <c r="AT123" s="5"/>
+      <c r="AU123" s="5"/>
+      <c r="AV123" s="5"/>
+      <c r="AW123" s="5"/>
+      <c r="AX123" s="5"/>
+      <c r="AY123" s="5"/>
+      <c r="AZ123" s="5"/>
+      <c r="BA123" s="5"/>
+      <c r="BB123" s="5"/>
+      <c r="BC123" s="5"/>
+      <c r="BD123" s="5"/>
+      <c r="BE123" s="5"/>
+      <c r="BF123" s="5"/>
+      <c r="BG123" s="5"/>
+      <c r="BH123" s="5"/>
+      <c r="BI123" s="5"/>
+      <c r="BJ123" s="5"/>
+      <c r="BK123" s="5"/>
+      <c r="BL123" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="BM123" s="5"/>
+      <c r="BN123" s="5"/>
+      <c r="BO123" s="5"/>
+      <c r="BP123" s="5"/>
+      <c r="BQ123" s="5"/>
+      <c r="BR123" s="5"/>
+      <c r="BS123" s="5"/>
+      <c r="BT123" s="5"/>
+      <c r="BU123" s="5"/>
+      <c r="BV123" s="5"/>
+      <c r="BW123" s="5"/>
+      <c r="BX123" s="5"/>
+      <c r="BY123" s="5"/>
+      <c r="BZ123" s="5"/>
+      <c r="CA123" s="5"/>
+      <c r="CB123" s="5"/>
+      <c r="CC123" s="5"/>
+      <c r="CD123" s="5"/>
+      <c r="CE123" s="5"/>
+      <c r="CF123" s="5"/>
     </row>
-    <row r="120" ht="26" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A120" s="6"/>
-      <c r="B120" s="6"/>
-      <c r="C120" s="6"/>
-      <c r="D120" s="6"/>
-      <c r="E120" s="6"/>
-      <c r="F120" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="G120" s="5"/>
-      <c r="H120" s="5"/>
-      <c r="I120" s="5"/>
-      <c r="J120" s="5"/>
-      <c r="K120" s="5"/>
-      <c r="L120" s="5"/>
-      <c r="M120" s="5"/>
-      <c r="N120" s="5"/>
-      <c r="O120" s="5"/>
-      <c r="P120" s="5"/>
-      <c r="Q120" s="5"/>
-      <c r="R120" s="5"/>
-      <c r="S120" s="7"/>
-      <c r="T120" s="7"/>
-      <c r="U120" s="7"/>
-      <c r="V120" s="6"/>
-      <c r="W120" s="6"/>
-      <c r="X120" s="6"/>
-      <c r="Y120" s="6"/>
-      <c r="Z120" s="6"/>
-      <c r="AA120" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="AB120" s="5"/>
-      <c r="AC120" s="5"/>
-      <c r="AD120" s="5"/>
-      <c r="AE120" s="5"/>
-      <c r="AF120" s="5"/>
-      <c r="AG120" s="5"/>
-      <c r="AH120" s="5"/>
-      <c r="AI120" s="5"/>
-      <c r="AJ120" s="5"/>
-      <c r="AK120" s="5"/>
-      <c r="AL120" s="5"/>
-      <c r="AM120" s="5"/>
-      <c r="AN120" s="7"/>
-      <c r="AO120" s="7"/>
-      <c r="AP120" s="7"/>
-      <c r="AQ120" s="6">
-        <v>46023</v>
-      </c>
-      <c r="AR120" s="6"/>
-      <c r="AS120" s="6"/>
-      <c r="AT120" s="6"/>
-      <c r="AU120" s="6"/>
-      <c r="AV120" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="AW120" s="5"/>
-      <c r="AX120" s="5"/>
-      <c r="AY120" s="5"/>
-      <c r="AZ120" s="5"/>
-      <c r="BA120" s="5"/>
-      <c r="BB120" s="5"/>
-      <c r="BC120" s="5"/>
-      <c r="BD120" s="5"/>
-      <c r="BE120" s="5"/>
-      <c r="BF120" s="5"/>
-      <c r="BG120" s="5"/>
-      <c r="BH120" s="5"/>
-      <c r="BI120" s="7">
-        <v>150</v>
-      </c>
-      <c r="BJ120" s="7"/>
-      <c r="BK120" s="7"/>
-      <c r="BL120" s="6"/>
-      <c r="BM120" s="6"/>
-      <c r="BN120" s="6"/>
-      <c r="BO120" s="6"/>
-      <c r="BP120" s="6"/>
-      <c r="BQ120" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="BR120" s="5"/>
-      <c r="BS120" s="5"/>
-      <c r="BT120" s="5"/>
-      <c r="BU120" s="5"/>
-      <c r="BV120" s="5"/>
-      <c r="BW120" s="5"/>
-      <c r="BX120" s="5"/>
-      <c r="BY120" s="5"/>
-      <c r="BZ120" s="5"/>
-      <c r="CA120" s="5"/>
-      <c r="CB120" s="5"/>
-      <c r="CC120" s="5"/>
-      <c r="CD120" s="7"/>
-      <c r="CE120" s="7"/>
-      <c r="CF120" s="7"/>
+    <row r="125" ht="30" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
+      <c r="A125" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B125" s="2"/>
+      <c r="C125" s="2"/>
+      <c r="D125" s="2"/>
+      <c r="E125" s="2"/>
+      <c r="F125" s="2"/>
+      <c r="G125" s="2"/>
+      <c r="H125" s="2"/>
+      <c r="I125" s="2"/>
+      <c r="J125" s="2"/>
+      <c r="K125" s="2"/>
+      <c r="L125" s="2"/>
+      <c r="M125" s="2"/>
+      <c r="N125" s="2"/>
+      <c r="O125" s="2"/>
+      <c r="P125" s="2"/>
+      <c r="Q125" s="2"/>
+      <c r="R125" s="2"/>
+      <c r="S125" s="2"/>
+      <c r="T125" s="2"/>
+      <c r="U125" s="2"/>
+      <c r="V125" s="2"/>
+      <c r="W125" s="2"/>
+      <c r="X125" s="2"/>
+      <c r="Y125" s="2"/>
+      <c r="Z125" s="2"/>
+      <c r="AA125" s="2"/>
+      <c r="AB125" s="2"/>
+      <c r="AC125" s="2"/>
+      <c r="AD125" s="2"/>
+      <c r="AE125" s="2"/>
+      <c r="AF125" s="2"/>
+      <c r="AG125" s="2"/>
+      <c r="AH125" s="2"/>
+      <c r="AI125" s="2"/>
+      <c r="AJ125" s="2"/>
+      <c r="AK125" s="2"/>
+      <c r="AL125" s="2"/>
+      <c r="AM125" s="2"/>
+      <c r="AN125" s="2"/>
+      <c r="AO125" s="2"/>
+      <c r="AP125" s="2"/>
+      <c r="AQ125" s="2"/>
+      <c r="AR125" s="2"/>
+      <c r="AS125" s="2"/>
+      <c r="AT125" s="2"/>
+      <c r="AU125" s="2"/>
+      <c r="AV125" s="2"/>
+      <c r="AW125" s="2"/>
+      <c r="AX125" s="2"/>
+      <c r="AY125" s="2"/>
+      <c r="AZ125" s="2"/>
+      <c r="BA125" s="2"/>
+      <c r="BB125" s="2"/>
+      <c r="BC125" s="2"/>
+      <c r="BD125" s="2"/>
+      <c r="BE125" s="2"/>
+      <c r="BF125" s="2"/>
+      <c r="BG125" s="2"/>
+      <c r="BH125" s="2"/>
+      <c r="BI125" s="2"/>
+      <c r="BJ125" s="2"/>
+      <c r="BK125" s="2"/>
+      <c r="BL125" s="2"/>
+      <c r="BM125" s="2"/>
+      <c r="BN125" s="2"/>
+      <c r="BO125" s="2"/>
+      <c r="BP125" s="2"/>
+      <c r="BQ125" s="2"/>
+      <c r="BR125" s="2"/>
+      <c r="BS125" s="2"/>
+      <c r="BT125" s="2"/>
+      <c r="BU125" s="2"/>
+      <c r="BV125" s="2"/>
+      <c r="BW125" s="2"/>
+      <c r="BX125" s="2"/>
+      <c r="BY125" s="2"/>
+      <c r="BZ125" s="2"/>
+      <c r="CA125" s="2"/>
+      <c r="CB125" s="2"/>
+      <c r="CC125" s="2"/>
+      <c r="CD125" s="2"/>
+      <c r="CE125" s="2"/>
+      <c r="CF125" s="2"/>
     </row>
-    <row r="121" ht="26" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A121" s="10"/>
-      <c r="B121" s="10"/>
-      <c r="C121" s="10"/>
-      <c r="D121" s="10"/>
-      <c r="E121" s="10"/>
-      <c r="F121" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="G121" s="11"/>
-      <c r="H121" s="11"/>
-      <c r="I121" s="11"/>
-      <c r="J121" s="11"/>
-      <c r="K121" s="11"/>
-      <c r="L121" s="11"/>
-      <c r="M121" s="11"/>
-      <c r="N121" s="11"/>
-      <c r="O121" s="11"/>
-      <c r="P121" s="11"/>
-      <c r="Q121" s="11"/>
-      <c r="R121" s="11"/>
-      <c r="S121" s="12">
-        <v>500</v>
-      </c>
-      <c r="T121" s="12"/>
-      <c r="U121" s="12"/>
-      <c r="V121" s="10"/>
-      <c r="W121" s="10"/>
-      <c r="X121" s="10"/>
-      <c r="Y121" s="10"/>
-      <c r="Z121" s="10"/>
-      <c r="AA121" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="AB121" s="11"/>
-      <c r="AC121" s="11"/>
-      <c r="AD121" s="11"/>
-      <c r="AE121" s="11"/>
-      <c r="AF121" s="11"/>
-      <c r="AG121" s="11"/>
-      <c r="AH121" s="11"/>
-      <c r="AI121" s="11"/>
-      <c r="AJ121" s="11"/>
-      <c r="AK121" s="11"/>
-      <c r="AL121" s="11"/>
-      <c r="AM121" s="11"/>
-      <c r="AN121" s="12">
-        <v>250</v>
-      </c>
-      <c r="AO121" s="12"/>
-      <c r="AP121" s="12"/>
-      <c r="AQ121" s="6"/>
-      <c r="AR121" s="6"/>
-      <c r="AS121" s="6"/>
-      <c r="AT121" s="6"/>
-      <c r="AU121" s="6"/>
-      <c r="AV121" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="AW121" s="5"/>
-      <c r="AX121" s="5"/>
-      <c r="AY121" s="5"/>
-      <c r="AZ121" s="5"/>
-      <c r="BA121" s="5"/>
-      <c r="BB121" s="5"/>
-      <c r="BC121" s="5"/>
-      <c r="BD121" s="5"/>
-      <c r="BE121" s="5"/>
-      <c r="BF121" s="5"/>
-      <c r="BG121" s="5"/>
-      <c r="BH121" s="5"/>
-      <c r="BI121" s="7"/>
-      <c r="BJ121" s="7"/>
-      <c r="BK121" s="7"/>
-      <c r="BL121" s="10"/>
-      <c r="BM121" s="10"/>
-      <c r="BN121" s="10"/>
-      <c r="BO121" s="10"/>
-      <c r="BP121" s="10"/>
-      <c r="BQ121" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="BR121" s="11"/>
-      <c r="BS121" s="11"/>
-      <c r="BT121" s="11"/>
-      <c r="BU121" s="11"/>
-      <c r="BV121" s="11"/>
-      <c r="BW121" s="11"/>
-      <c r="BX121" s="11"/>
-      <c r="BY121" s="11"/>
-      <c r="BZ121" s="11"/>
-      <c r="CA121" s="11"/>
-      <c r="CB121" s="11"/>
-      <c r="CC121" s="11"/>
-      <c r="CD121" s="12">
-        <v>300</v>
-      </c>
-      <c r="CE121" s="12"/>
-      <c r="CF121" s="12"/>
-    </row>
-    <row r="122" ht="26" customHeight="1" spans="43:63" x14ac:dyDescent="0.25">
-      <c r="AQ122" s="6"/>
-      <c r="AR122" s="6"/>
-      <c r="AS122" s="6"/>
-      <c r="AT122" s="6"/>
-      <c r="AU122" s="6"/>
-      <c r="AV122" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="AW122" s="5"/>
-      <c r="AX122" s="5"/>
-      <c r="AY122" s="5"/>
-      <c r="AZ122" s="5"/>
-      <c r="BA122" s="5"/>
-      <c r="BB122" s="5"/>
-      <c r="BC122" s="5"/>
-      <c r="BD122" s="5"/>
-      <c r="BE122" s="5"/>
-      <c r="BF122" s="5"/>
-      <c r="BG122" s="5"/>
-      <c r="BH122" s="5"/>
-      <c r="BI122" s="7"/>
-      <c r="BJ122" s="7"/>
-      <c r="BK122" s="7"/>
-    </row>
-    <row r="123" ht="24" customHeight="1" spans="43:63" x14ac:dyDescent="0.25">
-      <c r="AQ123" s="10"/>
-      <c r="AR123" s="10"/>
-      <c r="AS123" s="10"/>
-      <c r="AT123" s="10"/>
-      <c r="AU123" s="10"/>
-      <c r="AV123" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="AW123" s="11"/>
-      <c r="AX123" s="11"/>
-      <c r="AY123" s="11"/>
-      <c r="AZ123" s="11"/>
-      <c r="BA123" s="11"/>
-      <c r="BB123" s="11"/>
-      <c r="BC123" s="11"/>
-      <c r="BD123" s="11"/>
-      <c r="BE123" s="11"/>
-      <c r="BF123" s="11"/>
-      <c r="BG123" s="11"/>
-      <c r="BH123" s="11"/>
-      <c r="BI123" s="12">
-        <v>550</v>
-      </c>
-      <c r="BJ123" s="12"/>
-      <c r="BK123" s="12"/>
-    </row>
-    <row r="125" ht="22" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A125" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="B125" s="3"/>
-      <c r="C125" s="3"/>
-      <c r="D125" s="3"/>
-      <c r="E125" s="3"/>
-      <c r="F125" s="3"/>
-      <c r="G125" s="3"/>
-      <c r="H125" s="3"/>
-      <c r="I125" s="3"/>
-      <c r="J125" s="3"/>
-      <c r="K125" s="3"/>
-      <c r="L125" s="3"/>
-      <c r="M125" s="3"/>
-      <c r="N125" s="3"/>
-      <c r="O125" s="3"/>
-      <c r="P125" s="3"/>
-      <c r="Q125" s="3"/>
-      <c r="R125" s="3"/>
-      <c r="S125" s="3"/>
-      <c r="T125" s="3"/>
-      <c r="U125" s="3"/>
-      <c r="V125" s="3"/>
-      <c r="W125" s="3"/>
-      <c r="X125" s="3"/>
-      <c r="Y125" s="3"/>
-      <c r="Z125" s="3"/>
-      <c r="AA125" s="3"/>
-      <c r="AB125" s="3"/>
-      <c r="AC125" s="3"/>
-      <c r="AD125" s="3"/>
-      <c r="AE125" s="3"/>
-      <c r="AF125" s="3"/>
-      <c r="AG125" s="3"/>
-      <c r="AH125" s="3"/>
-      <c r="AI125" s="3"/>
-      <c r="AJ125" s="3"/>
-      <c r="AK125" s="3"/>
-      <c r="AL125" s="3"/>
-      <c r="AM125" s="3"/>
-      <c r="AN125" s="3"/>
-      <c r="AO125" s="3"/>
-      <c r="AP125" s="3"/>
-      <c r="AQ125" s="3"/>
-      <c r="AR125" s="3"/>
-      <c r="AS125" s="3"/>
-      <c r="AT125" s="3"/>
-      <c r="AU125" s="3"/>
-      <c r="AV125" s="3"/>
-      <c r="AW125" s="3"/>
-      <c r="AX125" s="3"/>
-      <c r="AY125" s="3"/>
-      <c r="AZ125" s="3"/>
-      <c r="BA125" s="3"/>
-      <c r="BB125" s="3"/>
-      <c r="BC125" s="3"/>
-      <c r="BD125" s="3"/>
-      <c r="BE125" s="3"/>
-      <c r="BF125" s="3"/>
-      <c r="BG125" s="3"/>
-      <c r="BH125" s="3"/>
-      <c r="BI125" s="3"/>
-      <c r="BJ125" s="3"/>
-      <c r="BK125" s="3"/>
-      <c r="BL125" s="3"/>
-      <c r="BM125" s="3"/>
-      <c r="BN125" s="3"/>
-      <c r="BO125" s="3"/>
-      <c r="BP125" s="3"/>
-      <c r="BQ125" s="3"/>
-      <c r="BR125" s="3"/>
-      <c r="BS125" s="3"/>
-      <c r="BT125" s="3"/>
-      <c r="BU125" s="3"/>
-      <c r="BV125" s="3"/>
-      <c r="BW125" s="3"/>
-      <c r="BX125" s="3"/>
-      <c r="BY125" s="3"/>
-      <c r="BZ125" s="3"/>
-      <c r="CA125" s="3"/>
-      <c r="CB125" s="3"/>
-      <c r="CC125" s="3"/>
-      <c r="CD125" s="3"/>
-      <c r="CE125" s="3"/>
-      <c r="CF125" s="3"/>
-    </row>
-    <row r="126" ht="45" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A126" s="3" t="s">
+    <row r="126" ht="30" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
+      <c r="A126" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="B126" s="3"/>
-      <c r="C126" s="3"/>
-      <c r="D126" s="3"/>
-      <c r="E126" s="3"/>
-      <c r="F126" s="3"/>
-      <c r="G126" s="3"/>
-      <c r="H126" s="3"/>
-      <c r="I126" s="3"/>
-      <c r="J126" s="3"/>
-      <c r="K126" s="3"/>
-      <c r="L126" s="3"/>
-      <c r="M126" s="3"/>
-      <c r="N126" s="3"/>
-      <c r="O126" s="3"/>
-      <c r="P126" s="3"/>
-      <c r="Q126" s="3"/>
-      <c r="R126" s="3"/>
-      <c r="S126" s="3"/>
-      <c r="T126" s="3"/>
-      <c r="U126" s="3"/>
-      <c r="V126" s="3"/>
-      <c r="W126" s="3"/>
-      <c r="X126" s="3"/>
-      <c r="Y126" s="3"/>
-      <c r="Z126" s="3"/>
-      <c r="AA126" s="3"/>
-      <c r="AB126" s="3"/>
-      <c r="AC126" s="3"/>
-      <c r="AD126" s="3"/>
-      <c r="AE126" s="3"/>
-      <c r="AF126" s="3"/>
-      <c r="AG126" s="3"/>
-      <c r="AH126" s="3"/>
-      <c r="AI126" s="3"/>
-      <c r="AJ126" s="3"/>
-      <c r="AK126" s="3"/>
-      <c r="AL126" s="3"/>
-      <c r="AM126" s="3"/>
-      <c r="AN126" s="3"/>
-      <c r="AO126" s="3"/>
-      <c r="AP126" s="3"/>
-      <c r="AQ126" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="AR126" s="3"/>
-      <c r="AS126" s="3"/>
-      <c r="AT126" s="3"/>
-      <c r="AU126" s="3"/>
-      <c r="AV126" s="3"/>
-      <c r="AW126" s="3"/>
-      <c r="AX126" s="3"/>
-      <c r="AY126" s="3"/>
-      <c r="AZ126" s="3"/>
-      <c r="BA126" s="3"/>
-      <c r="BB126" s="3"/>
-      <c r="BC126" s="3"/>
-      <c r="BD126" s="3"/>
-      <c r="BE126" s="3"/>
-      <c r="BF126" s="3"/>
-      <c r="BG126" s="3"/>
-      <c r="BH126" s="3"/>
-      <c r="BI126" s="3"/>
-      <c r="BJ126" s="3"/>
-      <c r="BK126" s="3"/>
-      <c r="BL126" s="3"/>
-      <c r="BM126" s="3"/>
-      <c r="BN126" s="3"/>
-      <c r="BO126" s="3"/>
-      <c r="BP126" s="3"/>
-      <c r="BQ126" s="3"/>
-      <c r="BR126" s="3"/>
-      <c r="BS126" s="3"/>
-      <c r="BT126" s="3"/>
-      <c r="BU126" s="3"/>
-      <c r="BV126" s="3"/>
-      <c r="BW126" s="3"/>
-      <c r="BX126" s="3"/>
-      <c r="BY126" s="3"/>
-      <c r="BZ126" s="3"/>
-      <c r="CA126" s="3"/>
-      <c r="CB126" s="3"/>
-      <c r="CC126" s="3"/>
-      <c r="CD126" s="3"/>
-      <c r="CE126" s="3"/>
-      <c r="CF126" s="3"/>
-    </row>
-    <row r="127" ht="42" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A127" s="5"/>
-      <c r="B127" s="5"/>
-      <c r="C127" s="5"/>
-      <c r="D127" s="5"/>
-      <c r="E127" s="5"/>
-      <c r="F127" s="5"/>
-      <c r="G127" s="5"/>
-      <c r="H127" s="5"/>
-      <c r="I127" s="5"/>
-      <c r="J127" s="5"/>
-      <c r="K127" s="5"/>
-      <c r="L127" s="5"/>
-      <c r="M127" s="5"/>
-      <c r="N127" s="5"/>
-      <c r="O127" s="5"/>
-      <c r="P127" s="5"/>
-      <c r="Q127" s="5"/>
-      <c r="R127" s="5"/>
-      <c r="S127" s="5"/>
-      <c r="T127" s="5"/>
-      <c r="U127" s="5"/>
-      <c r="V127" s="5"/>
-      <c r="W127" s="5"/>
-      <c r="X127" s="5"/>
-      <c r="Y127" s="5"/>
-      <c r="Z127" s="5"/>
-      <c r="AA127" s="5"/>
-      <c r="AB127" s="5"/>
-      <c r="AC127" s="5"/>
-      <c r="AD127" s="5"/>
-      <c r="AE127" s="5"/>
-      <c r="AF127" s="5"/>
-      <c r="AG127" s="5"/>
-      <c r="AH127" s="5"/>
-      <c r="AI127" s="5"/>
-      <c r="AJ127" s="5"/>
-      <c r="AK127" s="5"/>
-      <c r="AL127" s="5"/>
-      <c r="AM127" s="5"/>
-      <c r="AN127" s="5"/>
-      <c r="AO127" s="5"/>
-      <c r="AP127" s="5"/>
-      <c r="AQ127" s="5"/>
-      <c r="AR127" s="5"/>
-      <c r="AS127" s="5"/>
-      <c r="AT127" s="5"/>
-      <c r="AU127" s="5"/>
-      <c r="AV127" s="5"/>
-      <c r="AW127" s="5"/>
-      <c r="AX127" s="5"/>
-      <c r="AY127" s="5"/>
-      <c r="AZ127" s="5"/>
-      <c r="BA127" s="5"/>
-      <c r="BB127" s="5"/>
-      <c r="BC127" s="5"/>
-      <c r="BD127" s="5"/>
-      <c r="BE127" s="5"/>
-      <c r="BF127" s="5"/>
-      <c r="BG127" s="5"/>
-      <c r="BH127" s="5"/>
-      <c r="BI127" s="5"/>
-      <c r="BJ127" s="5"/>
-      <c r="BK127" s="5"/>
-      <c r="BL127" s="5"/>
-      <c r="BM127" s="5"/>
-      <c r="BN127" s="5"/>
-      <c r="BO127" s="5"/>
-      <c r="BP127" s="5"/>
-      <c r="BQ127" s="5"/>
-      <c r="BR127" s="5"/>
-      <c r="BS127" s="5"/>
-      <c r="BT127" s="5"/>
-      <c r="BU127" s="5"/>
-      <c r="BV127" s="5"/>
-      <c r="BW127" s="5"/>
-      <c r="BX127" s="5"/>
-      <c r="BY127" s="5"/>
-      <c r="BZ127" s="5"/>
-      <c r="CA127" s="5"/>
-      <c r="CB127" s="5"/>
-      <c r="CC127" s="5"/>
-      <c r="CD127" s="5"/>
-      <c r="CE127" s="5"/>
-      <c r="CF127" s="5"/>
-    </row>
-    <row r="129" ht="30" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A129" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="B129" s="2"/>
-      <c r="C129" s="2"/>
-      <c r="D129" s="2"/>
-      <c r="E129" s="2"/>
-      <c r="F129" s="2"/>
-      <c r="G129" s="2"/>
-      <c r="H129" s="2"/>
-      <c r="I129" s="2"/>
-      <c r="J129" s="2"/>
-      <c r="K129" s="2"/>
-      <c r="L129" s="2"/>
-      <c r="M129" s="2"/>
-      <c r="N129" s="2"/>
-      <c r="O129" s="2"/>
-      <c r="P129" s="2"/>
-      <c r="Q129" s="2"/>
-      <c r="R129" s="2"/>
-      <c r="S129" s="2"/>
-      <c r="T129" s="2"/>
-      <c r="U129" s="2"/>
-      <c r="V129" s="2"/>
-      <c r="W129" s="2"/>
-      <c r="X129" s="2"/>
-      <c r="Y129" s="2"/>
-      <c r="Z129" s="2"/>
-      <c r="AA129" s="2"/>
-      <c r="AB129" s="2"/>
-      <c r="AC129" s="2"/>
-      <c r="AD129" s="2"/>
-      <c r="AE129" s="2"/>
-      <c r="AF129" s="2"/>
-      <c r="AG129" s="2"/>
-      <c r="AH129" s="2"/>
-      <c r="AI129" s="2"/>
-      <c r="AJ129" s="2"/>
-      <c r="AK129" s="2"/>
-      <c r="AL129" s="2"/>
-      <c r="AM129" s="2"/>
-      <c r="AN129" s="2"/>
-      <c r="AO129" s="2"/>
-      <c r="AP129" s="2"/>
-      <c r="AQ129" s="2"/>
-      <c r="AR129" s="2"/>
-      <c r="AS129" s="2"/>
-      <c r="AT129" s="2"/>
-      <c r="AU129" s="2"/>
-      <c r="AV129" s="2"/>
-      <c r="AW129" s="2"/>
-      <c r="AX129" s="2"/>
-      <c r="AY129" s="2"/>
-      <c r="AZ129" s="2"/>
-      <c r="BA129" s="2"/>
-      <c r="BB129" s="2"/>
-      <c r="BC129" s="2"/>
-      <c r="BD129" s="2"/>
-      <c r="BE129" s="2"/>
-      <c r="BF129" s="2"/>
-      <c r="BG129" s="2"/>
-      <c r="BH129" s="2"/>
-      <c r="BI129" s="2"/>
-      <c r="BJ129" s="2"/>
-      <c r="BK129" s="2"/>
-      <c r="BL129" s="2"/>
-      <c r="BM129" s="2"/>
-      <c r="BN129" s="2"/>
-      <c r="BO129" s="2"/>
-      <c r="BP129" s="2"/>
-      <c r="BQ129" s="2"/>
-      <c r="BR129" s="2"/>
-      <c r="BS129" s="2"/>
-      <c r="BT129" s="2"/>
-      <c r="BU129" s="2"/>
-      <c r="BV129" s="2"/>
-      <c r="BW129" s="2"/>
-      <c r="BX129" s="2"/>
-      <c r="BY129" s="2"/>
-      <c r="BZ129" s="2"/>
-      <c r="CA129" s="2"/>
-      <c r="CB129" s="2"/>
-      <c r="CC129" s="2"/>
-      <c r="CD129" s="2"/>
-      <c r="CE129" s="2"/>
-      <c r="CF129" s="2"/>
-    </row>
-    <row r="130" ht="30" customHeight="1" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A130" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="B130" s="2"/>
-      <c r="C130" s="2"/>
-      <c r="D130" s="2"/>
-      <c r="E130" s="2"/>
-      <c r="F130" s="2"/>
-      <c r="G130" s="2"/>
-      <c r="H130" s="2"/>
-      <c r="I130" s="2"/>
-      <c r="J130" s="2"/>
-      <c r="K130" s="2"/>
-      <c r="L130" s="2"/>
-      <c r="M130" s="2"/>
-      <c r="N130" s="2"/>
-      <c r="O130" s="2"/>
-      <c r="P130" s="2"/>
-      <c r="Q130" s="2"/>
-      <c r="R130" s="2"/>
-      <c r="S130" s="2"/>
-      <c r="T130" s="2"/>
-      <c r="U130" s="2"/>
-      <c r="V130" s="2"/>
-      <c r="W130" s="2"/>
-      <c r="X130" s="2"/>
-      <c r="Y130" s="2"/>
-      <c r="Z130" s="2"/>
-      <c r="AA130" s="2"/>
-      <c r="AB130" s="2"/>
-      <c r="AC130" s="2"/>
-      <c r="AD130" s="2"/>
-      <c r="AE130" s="2"/>
-      <c r="AF130" s="2"/>
-      <c r="AG130" s="2"/>
-      <c r="AH130" s="2"/>
-      <c r="AI130" s="2"/>
-      <c r="AJ130" s="2"/>
-      <c r="AK130" s="2"/>
-      <c r="AL130" s="2"/>
-      <c r="AM130" s="2"/>
-      <c r="AN130" s="2"/>
-      <c r="AO130" s="2"/>
-      <c r="AP130" s="2"/>
-      <c r="AQ130" s="2"/>
-      <c r="AR130" s="2"/>
-      <c r="AS130" s="2"/>
-      <c r="AT130" s="2"/>
-      <c r="AU130" s="2"/>
-      <c r="AV130" s="2"/>
-      <c r="AW130" s="2"/>
-      <c r="AX130" s="2"/>
-      <c r="AY130" s="2"/>
-      <c r="AZ130" s="2"/>
-      <c r="BA130" s="2"/>
-      <c r="BB130" s="2"/>
-      <c r="BC130" s="2"/>
-      <c r="BD130" s="2"/>
-      <c r="BE130" s="2"/>
-      <c r="BF130" s="2"/>
-      <c r="BG130" s="2"/>
-      <c r="BH130" s="2"/>
-      <c r="BI130" s="2"/>
-      <c r="BJ130" s="2"/>
-      <c r="BK130" s="2"/>
-      <c r="BL130" s="2"/>
-      <c r="BM130" s="2"/>
-      <c r="BN130" s="2"/>
-      <c r="BO130" s="2"/>
-      <c r="BP130" s="2"/>
-      <c r="BQ130" s="2"/>
-      <c r="BR130" s="2"/>
-      <c r="BS130" s="2"/>
-      <c r="BT130" s="2"/>
-      <c r="BU130" s="2"/>
-      <c r="BV130" s="2"/>
-      <c r="BW130" s="2"/>
-      <c r="BX130" s="2"/>
-      <c r="BY130" s="2"/>
-      <c r="BZ130" s="2"/>
-      <c r="CA130" s="2"/>
-      <c r="CB130" s="2"/>
-      <c r="CC130" s="2"/>
-      <c r="CD130" s="2"/>
-      <c r="CE130" s="2"/>
-      <c r="CF130" s="2"/>
+      <c r="B126" s="2"/>
+      <c r="C126" s="2"/>
+      <c r="D126" s="2"/>
+      <c r="E126" s="2"/>
+      <c r="F126" s="2"/>
+      <c r="G126" s="2"/>
+      <c r="H126" s="2"/>
+      <c r="I126" s="2"/>
+      <c r="J126" s="2"/>
+      <c r="K126" s="2"/>
+      <c r="L126" s="2"/>
+      <c r="M126" s="2"/>
+      <c r="N126" s="2"/>
+      <c r="O126" s="2"/>
+      <c r="P126" s="2"/>
+      <c r="Q126" s="2"/>
+      <c r="R126" s="2"/>
+      <c r="S126" s="2"/>
+      <c r="T126" s="2"/>
+      <c r="U126" s="2"/>
+      <c r="V126" s="2"/>
+      <c r="W126" s="2"/>
+      <c r="X126" s="2"/>
+      <c r="Y126" s="2"/>
+      <c r="Z126" s="2"/>
+      <c r="AA126" s="2"/>
+      <c r="AB126" s="2"/>
+      <c r="AC126" s="2"/>
+      <c r="AD126" s="2"/>
+      <c r="AE126" s="2"/>
+      <c r="AF126" s="2"/>
+      <c r="AG126" s="2"/>
+      <c r="AH126" s="2"/>
+      <c r="AI126" s="2"/>
+      <c r="AJ126" s="2"/>
+      <c r="AK126" s="2"/>
+      <c r="AL126" s="2"/>
+      <c r="AM126" s="2"/>
+      <c r="AN126" s="2"/>
+      <c r="AO126" s="2"/>
+      <c r="AP126" s="2"/>
+      <c r="AQ126" s="2"/>
+      <c r="AR126" s="2"/>
+      <c r="AS126" s="2"/>
+      <c r="AT126" s="2"/>
+      <c r="AU126" s="2"/>
+      <c r="AV126" s="2"/>
+      <c r="AW126" s="2"/>
+      <c r="AX126" s="2"/>
+      <c r="AY126" s="2"/>
+      <c r="AZ126" s="2"/>
+      <c r="BA126" s="2"/>
+      <c r="BB126" s="2"/>
+      <c r="BC126" s="2"/>
+      <c r="BD126" s="2"/>
+      <c r="BE126" s="2"/>
+      <c r="BF126" s="2"/>
+      <c r="BG126" s="2"/>
+      <c r="BH126" s="2"/>
+      <c r="BI126" s="2"/>
+      <c r="BJ126" s="2"/>
+      <c r="BK126" s="2"/>
+      <c r="BL126" s="2"/>
+      <c r="BM126" s="2"/>
+      <c r="BN126" s="2"/>
+      <c r="BO126" s="2"/>
+      <c r="BP126" s="2"/>
+      <c r="BQ126" s="2"/>
+      <c r="BR126" s="2"/>
+      <c r="BS126" s="2"/>
+      <c r="BT126" s="2"/>
+      <c r="BU126" s="2"/>
+      <c r="BV126" s="2"/>
+      <c r="BW126" s="2"/>
+      <c r="BX126" s="2"/>
+      <c r="BY126" s="2"/>
+      <c r="BZ126" s="2"/>
+      <c r="CA126" s="2"/>
+      <c r="CB126" s="2"/>
+      <c r="CC126" s="2"/>
+      <c r="CD126" s="2"/>
+      <c r="CE126" s="2"/>
+      <c r="CF126" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="1658">
+  <mergeCells count="1651">
     <mergeCell ref="A1:CF1"/>
     <mergeCell ref="A2:CF2"/>
     <mergeCell ref="A3:CF3"/>
@@ -14214,86 +13949,79 @@
     <mergeCell ref="BQ111:BV111"/>
     <mergeCell ref="BW111:CA111"/>
     <mergeCell ref="CB111:CF111"/>
-    <mergeCell ref="A113:CF113"/>
-    <mergeCell ref="A114:Q114"/>
-    <mergeCell ref="R114:AH114"/>
-    <mergeCell ref="AI114:AX114"/>
-    <mergeCell ref="AY114:BO114"/>
-    <mergeCell ref="BP114:CF114"/>
-    <mergeCell ref="A115:Q115"/>
-    <mergeCell ref="R115:AH115"/>
-    <mergeCell ref="AI115:AX115"/>
-    <mergeCell ref="AY115:BO115"/>
-    <mergeCell ref="BP115:CF115"/>
-    <mergeCell ref="A117:U117"/>
-    <mergeCell ref="V117:AP117"/>
-    <mergeCell ref="AQ117:BK117"/>
-    <mergeCell ref="BL117:CF117"/>
-    <mergeCell ref="A118:E118"/>
-    <mergeCell ref="F118:R118"/>
-    <mergeCell ref="S118:U118"/>
-    <mergeCell ref="V118:Z118"/>
-    <mergeCell ref="AA118:AM118"/>
-    <mergeCell ref="AN118:AP118"/>
-    <mergeCell ref="AQ118:AU118"/>
-    <mergeCell ref="AV118:BH118"/>
-    <mergeCell ref="BI118:BK118"/>
-    <mergeCell ref="BL118:BP118"/>
-    <mergeCell ref="BQ118:CC118"/>
-    <mergeCell ref="CD118:CF118"/>
-    <mergeCell ref="A119:E119"/>
-    <mergeCell ref="F119:R119"/>
-    <mergeCell ref="S119:U119"/>
-    <mergeCell ref="V119:Z119"/>
-    <mergeCell ref="AA119:AM119"/>
-    <mergeCell ref="AN119:AP119"/>
-    <mergeCell ref="AQ119:AU119"/>
-    <mergeCell ref="AV119:BH119"/>
-    <mergeCell ref="BI119:BK119"/>
-    <mergeCell ref="BL119:BP119"/>
-    <mergeCell ref="BQ119:CC119"/>
-    <mergeCell ref="CD119:CF119"/>
-    <mergeCell ref="A120:E120"/>
-    <mergeCell ref="F120:R120"/>
-    <mergeCell ref="S120:U120"/>
-    <mergeCell ref="V120:Z120"/>
-    <mergeCell ref="AA120:AM120"/>
-    <mergeCell ref="AN120:AP120"/>
-    <mergeCell ref="AQ120:AU120"/>
-    <mergeCell ref="AV120:BH120"/>
-    <mergeCell ref="BI120:BK120"/>
-    <mergeCell ref="BL120:BP120"/>
-    <mergeCell ref="BQ120:CC120"/>
-    <mergeCell ref="CD120:CF120"/>
-    <mergeCell ref="A121:E121"/>
-    <mergeCell ref="F121:R121"/>
-    <mergeCell ref="S121:U121"/>
-    <mergeCell ref="V121:Z121"/>
-    <mergeCell ref="AA121:AM121"/>
-    <mergeCell ref="AN121:AP121"/>
-    <mergeCell ref="AQ121:AU121"/>
-    <mergeCell ref="AV121:BH121"/>
-    <mergeCell ref="BI121:BK121"/>
-    <mergeCell ref="BL121:BP121"/>
-    <mergeCell ref="BQ121:CC121"/>
-    <mergeCell ref="CD121:CF121"/>
-    <mergeCell ref="AQ122:AU122"/>
-    <mergeCell ref="AV122:BH122"/>
-    <mergeCell ref="BI122:BK122"/>
-    <mergeCell ref="AQ123:AU123"/>
-    <mergeCell ref="AV123:BH123"/>
-    <mergeCell ref="BI123:BK123"/>
+    <mergeCell ref="A113:U113"/>
+    <mergeCell ref="V113:AP113"/>
+    <mergeCell ref="AQ113:BK113"/>
+    <mergeCell ref="BL113:CF113"/>
+    <mergeCell ref="A114:F114"/>
+    <mergeCell ref="G114:P114"/>
+    <mergeCell ref="Q114:U114"/>
+    <mergeCell ref="V114:AA114"/>
+    <mergeCell ref="AB114:AK114"/>
+    <mergeCell ref="AL114:AP114"/>
+    <mergeCell ref="AQ114:AV114"/>
+    <mergeCell ref="AW114:BF114"/>
+    <mergeCell ref="BG114:BK114"/>
+    <mergeCell ref="BL114:BQ114"/>
+    <mergeCell ref="BR114:CA114"/>
+    <mergeCell ref="CB114:CF114"/>
+    <mergeCell ref="A115:F115"/>
+    <mergeCell ref="G115:P115"/>
+    <mergeCell ref="Q115:U115"/>
+    <mergeCell ref="V115:AA115"/>
+    <mergeCell ref="AB115:AK115"/>
+    <mergeCell ref="AL115:AP115"/>
+    <mergeCell ref="AQ115:AV115"/>
+    <mergeCell ref="AW115:BF115"/>
+    <mergeCell ref="BG115:BK115"/>
+    <mergeCell ref="BL115:BQ115"/>
+    <mergeCell ref="BR115:CA115"/>
+    <mergeCell ref="CB115:CF115"/>
+    <mergeCell ref="A116:F116"/>
+    <mergeCell ref="G116:P116"/>
+    <mergeCell ref="Q116:U116"/>
+    <mergeCell ref="V116:AA116"/>
+    <mergeCell ref="AB116:AK116"/>
+    <mergeCell ref="AL116:AP116"/>
+    <mergeCell ref="AQ116:AV116"/>
+    <mergeCell ref="AW116:BF116"/>
+    <mergeCell ref="BG116:BK116"/>
+    <mergeCell ref="BL116:BQ116"/>
+    <mergeCell ref="BR116:CA116"/>
+    <mergeCell ref="CB116:CF116"/>
+    <mergeCell ref="A117:F117"/>
+    <mergeCell ref="G117:P117"/>
+    <mergeCell ref="Q117:U117"/>
+    <mergeCell ref="V117:AA117"/>
+    <mergeCell ref="AB117:AK117"/>
+    <mergeCell ref="AL117:AP117"/>
+    <mergeCell ref="AQ117:AV117"/>
+    <mergeCell ref="AW117:BF117"/>
+    <mergeCell ref="BG117:BK117"/>
+    <mergeCell ref="BL117:BQ117"/>
+    <mergeCell ref="BR117:CA117"/>
+    <mergeCell ref="CB117:CF117"/>
+    <mergeCell ref="AQ118:AV118"/>
+    <mergeCell ref="AW118:BF118"/>
+    <mergeCell ref="BG118:BK118"/>
+    <mergeCell ref="AQ119:AV119"/>
+    <mergeCell ref="AW119:BF119"/>
+    <mergeCell ref="BG119:BK119"/>
+    <mergeCell ref="A121:CF121"/>
+    <mergeCell ref="A122:U122"/>
+    <mergeCell ref="V122:AP122"/>
+    <mergeCell ref="AQ122:BK122"/>
+    <mergeCell ref="BL122:CF122"/>
+    <mergeCell ref="A123:U123"/>
+    <mergeCell ref="V123:AP123"/>
+    <mergeCell ref="AQ123:BK123"/>
+    <mergeCell ref="BL123:CF123"/>
     <mergeCell ref="A125:CF125"/>
-    <mergeCell ref="A126:AP126"/>
-    <mergeCell ref="AQ126:CF126"/>
-    <mergeCell ref="A127:AP127"/>
-    <mergeCell ref="AQ127:CF127"/>
-    <mergeCell ref="A129:CF129"/>
-    <mergeCell ref="A130:CF130"/>
+    <mergeCell ref="A126:CF126"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.1" footer="0.1"/>
-  <pageSetup paperSize="8" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
   <headerFooter>
     <oddFooter>&amp;LGujjar Brother Transport&amp;RPAGE &amp;P / &amp;N</oddFooter>
   </headerFooter>

</xml_diff>